<commit_message>
Checkpoint: Series A cap table complete
</commit_message>
<xml_diff>
--- a/runs/20260415-101320/models/model.xlsx
+++ b/runs/20260415-101320/models/model.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/var/folders/pk/d3fxz1r57v334zbrzvw1g9pw0000gn/T/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{648287A4-AFC4-1C42-8A53-ED78325E6B96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{02EECB1D-FB7C-6543-8B1A-FB812B9D510C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="__temp__" sheetId="152" r:id="rId1"/>
     <sheet name="DetailedCapTable" sheetId="153" r:id="rId2"/>
     <sheet name="SAFE Investments" sheetId="154" r:id="rId3"/>
+    <sheet name="Series A" sheetId="155" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029" iterate="1"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="88">
   <si>
     <t>Total</t>
   </si>
@@ -193,17 +194,125 @@
     <t>Mark Lotke</t>
   </si>
   <si>
+    <t>SIDEKICK (THINK MORE SECURITY, INC.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Common </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Option </t>
+  </si>
+  <si>
+    <t>Series A</t>
+  </si>
+  <si>
+    <t>Total Capitalization</t>
+  </si>
+  <si>
+    <t># of</t>
+  </si>
+  <si>
+    <t>$</t>
+  </si>
+  <si>
+    <t>Preferred</t>
+  </si>
+  <si>
+    <t>Pool +</t>
+  </si>
+  <si>
+    <t>Total FD</t>
+  </si>
+  <si>
+    <t>Shares</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Invested</t>
+  </si>
+  <si>
+    <t>Pre A</t>
+  </si>
+  <si>
+    <t>FD</t>
+  </si>
+  <si>
+    <t>Common Stock and Options:</t>
+  </si>
+  <si>
+    <t>Total Common</t>
+  </si>
+  <si>
+    <t>Preferred Rounds</t>
+  </si>
+  <si>
+    <t>Elizabeth A. Donaghey</t>
+  </si>
+  <si>
+    <t>Totals</t>
+  </si>
+  <si>
+    <t>Price per Share</t>
+  </si>
+  <si>
+    <t>Pre-Money Valuation</t>
+  </si>
+  <si>
+    <t>Post-Money Valuation</t>
+  </si>
+  <si>
+    <t>Series A Assumptions:</t>
+  </si>
+  <si>
+    <t>Total Raised</t>
+  </si>
+  <si>
+    <t>Pre-Money Valuation Step-up</t>
+  </si>
+  <si>
+    <t>Pre SAFE</t>
+  </si>
+  <si>
+    <t>Other Common Shareholders</t>
+  </si>
+  <si>
+    <t>ESOP Available</t>
+  </si>
+  <si>
+    <t>Other SAFE Investors</t>
+  </si>
+  <si>
+    <t>Other Series A</t>
+  </si>
+  <si>
+    <t>Option Pool Expansion</t>
+  </si>
+  <si>
     <t>Transfer from Owl Rocl Capital II, LLC (Accomplice)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% </t>
+  </si>
+  <si>
+    <t>% Ownership (Series A)</t>
+  </si>
+  <si>
+    <t>SIDEKICK &amp; TEN ELEVEN SERIES A</t>
+  </si>
+  <si>
+    <t>Ten Eleven Ventures</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="4">
+    <numFmt numFmtId="5" formatCode="&quot;$&quot;#,##0_);\(&quot;$&quot;#,##0\)"/>
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="175" formatCode="_-[$$-409]* #,##0.0000_-;_-[$$-409]* \(#,##0.0000\)_-;_-[$$-409]* &quot;-&quot;??;_-@_-"/>
   </numFmts>
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="28" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -339,6 +448,37 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF008000"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
+    <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
@@ -364,8 +504,15 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -545,8 +692,14 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="24">
     <border>
       <left/>
       <right/>
@@ -661,6 +814,156 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -706,35 +1009,99 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="165" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="19" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="37" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="37" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="5" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="175" fontId="22" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="5" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="5" fontId="18" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="18" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="37" fontId="18" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="37" fontId="18" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="5" fontId="18" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="18" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1155,610 +1522,610 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
+      <c r="A1" s="5"/>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="5"/>
+      <c r="J1" s="5"/>
+      <c r="K1" s="5"/>
+      <c r="L1" s="5"/>
+      <c r="M1" s="5"/>
+      <c r="N1" s="5"/>
+      <c r="O1" s="5"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="4" t="s">
+      <c r="A2" s="5"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
-      <c r="N2" s="1"/>
-      <c r="O2" s="1"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="5"/>
+      <c r="L2" s="5"/>
+      <c r="M2" s="5"/>
+      <c r="N2" s="5"/>
+      <c r="O2" s="5"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A3" s="1"/>
-      <c r="B3" s="4" t="s">
+      <c r="A3" s="5"/>
+      <c r="B3" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="16" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="16" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
-      <c r="L3" s="1"/>
-      <c r="M3" s="1"/>
-      <c r="N3" s="1"/>
-      <c r="O3" s="1"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
+      <c r="N3" s="5"/>
+      <c r="O3" s="5"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A4" s="1"/>
-      <c r="B4" s="3" t="s">
+      <c r="A4" s="5"/>
+      <c r="B4" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4" s="32">
         <v>3600000</v>
       </c>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7">
+      <c r="D4" s="32"/>
+      <c r="E4" s="32"/>
+      <c r="F4" s="32"/>
+      <c r="G4" s="32">
         <f>SUM(C4:F4)</f>
         <v>3600000</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="6">
         <f>G4/$G$23</f>
         <v>0.36959987630724139</v>
       </c>
-      <c r="I4" s="2"/>
-      <c r="J4" s="1"/>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
-      <c r="M4" s="1"/>
-      <c r="N4" s="1"/>
-      <c r="O4" s="1"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="5"/>
+      <c r="K4" s="5"/>
+      <c r="L4" s="5"/>
+      <c r="M4" s="5"/>
+      <c r="N4" s="5"/>
+      <c r="O4" s="5"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A5" s="1"/>
-      <c r="B5" s="3" t="s">
+      <c r="A5" s="5"/>
+      <c r="B5" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="7">
+      <c r="C5" s="32">
         <v>3600000</v>
       </c>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7">
+      <c r="D5" s="32"/>
+      <c r="E5" s="32"/>
+      <c r="F5" s="32"/>
+      <c r="G5" s="32">
         <f>SUM(C5:F5)</f>
         <v>3600000</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="6">
         <f>G5/$G$23</f>
         <v>0.36959987630724139</v>
       </c>
-      <c r="I5" s="2"/>
-      <c r="J5" s="1"/>
-      <c r="K5" s="1"/>
-      <c r="L5" s="1"/>
-      <c r="M5" s="1"/>
-      <c r="N5" s="1"/>
-      <c r="O5" s="1"/>
+      <c r="I5" s="6"/>
+      <c r="J5" s="5"/>
+      <c r="K5" s="5"/>
+      <c r="L5" s="5"/>
+      <c r="M5" s="5"/>
+      <c r="N5" s="5"/>
+      <c r="O5" s="5"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A6" s="1"/>
-      <c r="B6" s="3" t="s">
+      <c r="A6" s="5"/>
+      <c r="B6" s="15" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="7">
+      <c r="C6" s="32">
         <v>222187</v>
       </c>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7">
+      <c r="D6" s="32"/>
+      <c r="E6" s="32"/>
+      <c r="F6" s="32"/>
+      <c r="G6" s="32">
         <f>SUM(C6:F6)</f>
         <v>222187</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="6">
         <f>G6/$G$23</f>
         <v>2.28111910325214E-2</v>
       </c>
-      <c r="I6" s="2"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
-      <c r="L6" s="1"/>
-      <c r="M6" s="1"/>
-      <c r="N6" s="1"/>
-      <c r="O6" s="1"/>
+      <c r="I6" s="6"/>
+      <c r="J6" s="5"/>
+      <c r="K6" s="5"/>
+      <c r="L6" s="5"/>
+      <c r="M6" s="5"/>
+      <c r="N6" s="5"/>
+      <c r="O6" s="5"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A7" s="1"/>
-      <c r="B7" s="3" t="s">
+      <c r="A7" s="5"/>
+      <c r="B7" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="7">
+      <c r="C7" s="32">
         <v>592500</v>
       </c>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7">
+      <c r="D7" s="32"/>
+      <c r="E7" s="32"/>
+      <c r="F7" s="32"/>
+      <c r="G7" s="32">
         <f>SUM(C7:F7)</f>
         <v>592500</v>
       </c>
-      <c r="H7" s="2">
+      <c r="H7" s="6">
         <f>G7/$G$23</f>
         <v>6.0829979642233481E-2</v>
       </c>
-      <c r="I7" s="2"/>
-      <c r="J7" s="1"/>
-      <c r="K7" s="1"/>
-      <c r="L7" s="1"/>
-      <c r="M7" s="1"/>
-      <c r="N7" s="1"/>
-      <c r="O7" s="1"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="5"/>
+      <c r="K7" s="5"/>
+      <c r="L7" s="5"/>
+      <c r="M7" s="5"/>
+      <c r="N7" s="5"/>
+      <c r="O7" s="5"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A8" s="1"/>
-      <c r="B8" s="3" t="s">
+      <c r="A8" s="5"/>
+      <c r="B8" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="7">
+      <c r="C8" s="32">
         <v>592500</v>
       </c>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7">
+      <c r="D8" s="32"/>
+      <c r="E8" s="32"/>
+      <c r="F8" s="32"/>
+      <c r="G8" s="32">
         <f>SUM(C8:F8)</f>
         <v>592500</v>
       </c>
-      <c r="H8" s="2">
+      <c r="H8" s="6">
         <f>G8/$G$23</f>
         <v>6.0829979642233481E-2</v>
       </c>
-      <c r="I8" s="2"/>
-      <c r="J8" s="1"/>
-      <c r="K8" s="1"/>
-      <c r="L8" s="1"/>
-      <c r="M8" s="1"/>
-      <c r="N8" s="1"/>
-      <c r="O8" s="1"/>
+      <c r="I8" s="6"/>
+      <c r="J8" s="5"/>
+      <c r="K8" s="5"/>
+      <c r="L8" s="5"/>
+      <c r="M8" s="5"/>
+      <c r="N8" s="5"/>
+      <c r="O8" s="5"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A9" s="1"/>
-      <c r="B9" s="3" t="s">
+      <c r="A9" s="5"/>
+      <c r="B9" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="7">
+      <c r="C9" s="32">
         <v>13500</v>
       </c>
-      <c r="D9" s="7">
+      <c r="D9" s="32">
         <v>98900</v>
       </c>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7">
+      <c r="E9" s="32"/>
+      <c r="F9" s="32"/>
+      <c r="G9" s="32">
         <f>SUM(C9:F9)</f>
         <v>112400</v>
       </c>
-      <c r="H9" s="2">
+      <c r="H9" s="6">
         <f>G9/$G$23</f>
         <v>1.1539729471370537E-2</v>
       </c>
-      <c r="I9" s="2"/>
-      <c r="J9" s="1"/>
-      <c r="K9" s="1"/>
-      <c r="L9" s="1"/>
-      <c r="M9" s="1"/>
-      <c r="N9" s="1"/>
-      <c r="O9" s="1"/>
+      <c r="I9" s="6"/>
+      <c r="J9" s="5"/>
+      <c r="K9" s="5"/>
+      <c r="L9" s="5"/>
+      <c r="M9" s="5"/>
+      <c r="N9" s="5"/>
+      <c r="O9" s="5"/>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A10" s="1"/>
-      <c r="B10" s="3" t="s">
+      <c r="A10" s="5"/>
+      <c r="B10" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="7">
+      <c r="C10" s="32">
         <v>9000</v>
       </c>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7">
+      <c r="D10" s="32"/>
+      <c r="E10" s="32"/>
+      <c r="F10" s="32"/>
+      <c r="G10" s="32">
         <f>SUM(C10:F10)</f>
         <v>9000</v>
       </c>
-      <c r="H10" s="2">
+      <c r="H10" s="6">
         <f>G10/$G$23</f>
         <v>9.2399969076810353E-4</v>
       </c>
-      <c r="I10" s="2"/>
-      <c r="J10" s="1"/>
-      <c r="K10" s="1"/>
-      <c r="L10" s="1"/>
-      <c r="M10" s="1"/>
-      <c r="N10" s="1"/>
-      <c r="O10" s="1"/>
+      <c r="I10" s="6"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+      <c r="L10" s="5"/>
+      <c r="M10" s="5"/>
+      <c r="N10" s="5"/>
+      <c r="O10" s="5"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A11" s="1"/>
-      <c r="B11" s="3" t="s">
+      <c r="A11" s="5"/>
+      <c r="B11" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7">
+      <c r="C11" s="32"/>
+      <c r="D11" s="32">
         <v>95000</v>
       </c>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7">
+      <c r="E11" s="32"/>
+      <c r="F11" s="32"/>
+      <c r="G11" s="32">
         <f>SUM(C11:F11)</f>
         <v>95000</v>
       </c>
-      <c r="H11" s="2">
+      <c r="H11" s="6">
         <f>G11/$G$23</f>
         <v>9.7533300692188695E-3</v>
       </c>
-      <c r="I11" s="2"/>
-      <c r="J11" s="1"/>
-      <c r="K11" s="1"/>
-      <c r="L11" s="1"/>
-      <c r="M11" s="1"/>
-      <c r="N11" s="1"/>
-      <c r="O11" s="1"/>
+      <c r="I11" s="6"/>
+      <c r="J11" s="5"/>
+      <c r="K11" s="5"/>
+      <c r="L11" s="5"/>
+      <c r="M11" s="5"/>
+      <c r="N11" s="5"/>
+      <c r="O11" s="5"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A12" s="1"/>
-      <c r="B12" s="3" t="s">
+      <c r="A12" s="5"/>
+      <c r="B12" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7">
+      <c r="C12" s="32"/>
+      <c r="D12" s="32"/>
+      <c r="E12" s="32">
         <v>25000</v>
       </c>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7">
+      <c r="F12" s="32"/>
+      <c r="G12" s="32">
         <f>SUM(C12:F12)</f>
         <v>25000</v>
       </c>
-      <c r="H12" s="2">
+      <c r="H12" s="6">
         <f>G12/$G$23</f>
         <v>2.5666658076891765E-3</v>
       </c>
-      <c r="I12" s="2"/>
-      <c r="J12" s="1"/>
-      <c r="K12" s="1"/>
-      <c r="L12" s="1"/>
-      <c r="M12" s="1"/>
-      <c r="N12" s="1"/>
-      <c r="O12" s="1"/>
+      <c r="I12" s="6"/>
+      <c r="J12" s="5"/>
+      <c r="K12" s="5"/>
+      <c r="L12" s="5"/>
+      <c r="M12" s="5"/>
+      <c r="N12" s="5"/>
+      <c r="O12" s="5"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A13" s="1"/>
-      <c r="B13" s="3" t="s">
+      <c r="A13" s="5"/>
+      <c r="B13" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7">
+      <c r="C13" s="32"/>
+      <c r="D13" s="32"/>
+      <c r="E13" s="32">
         <v>41562</v>
       </c>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7">
+      <c r="F13" s="32"/>
+      <c r="G13" s="32">
         <f>SUM(C13:F13)</f>
         <v>41562</v>
       </c>
-      <c r="H13" s="2">
+      <c r="H13" s="6">
         <f>G13/$G$23</f>
         <v>4.2670305719671019E-3</v>
       </c>
-      <c r="I13" s="2"/>
-      <c r="J13" s="1"/>
-      <c r="K13" s="1"/>
-      <c r="L13" s="1"/>
-      <c r="M13" s="1"/>
-      <c r="N13" s="1"/>
-      <c r="O13" s="1"/>
+      <c r="I13" s="6"/>
+      <c r="J13" s="5"/>
+      <c r="K13" s="5"/>
+      <c r="L13" s="5"/>
+      <c r="M13" s="5"/>
+      <c r="N13" s="5"/>
+      <c r="O13" s="5"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A14" s="1"/>
-      <c r="B14" s="3" t="s">
+      <c r="A14" s="5"/>
+      <c r="B14" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7">
+      <c r="C14" s="32"/>
+      <c r="D14" s="32">
         <v>285000</v>
       </c>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="7">
+      <c r="E14" s="32"/>
+      <c r="F14" s="32"/>
+      <c r="G14" s="32">
         <f>SUM(C14:F14)</f>
         <v>285000</v>
       </c>
-      <c r="H14" s="2">
+      <c r="H14" s="6">
         <f>G14/$G$23</f>
         <v>2.925999020765661E-2</v>
       </c>
-      <c r="I14" s="2"/>
-      <c r="J14" s="1"/>
-      <c r="K14" s="1"/>
-      <c r="L14" s="1"/>
-      <c r="M14" s="1"/>
-      <c r="N14" s="1"/>
-      <c r="O14" s="1"/>
+      <c r="I14" s="6"/>
+      <c r="J14" s="5"/>
+      <c r="K14" s="5"/>
+      <c r="L14" s="5"/>
+      <c r="M14" s="5"/>
+      <c r="N14" s="5"/>
+      <c r="O14" s="5"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A15" s="1"/>
-      <c r="B15" s="3" t="s">
+      <c r="A15" s="5"/>
+      <c r="B15" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7">
+      <c r="C15" s="32"/>
+      <c r="D15" s="32">
         <v>50000</v>
       </c>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="7">
+      <c r="E15" s="32"/>
+      <c r="F15" s="32"/>
+      <c r="G15" s="32">
         <f>SUM(C15:F15)</f>
         <v>50000</v>
       </c>
-      <c r="H15" s="2">
+      <c r="H15" s="6">
         <f>G15/$G$23</f>
         <v>5.133331615378353E-3</v>
       </c>
-      <c r="I15" s="2"/>
-      <c r="J15" s="1"/>
-      <c r="K15" s="1"/>
-      <c r="L15" s="1"/>
-      <c r="M15" s="1"/>
-      <c r="N15" s="1"/>
-      <c r="O15" s="1"/>
+      <c r="I15" s="6"/>
+      <c r="J15" s="5"/>
+      <c r="K15" s="5"/>
+      <c r="L15" s="5"/>
+      <c r="M15" s="5"/>
+      <c r="N15" s="5"/>
+      <c r="O15" s="5"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A16" s="1"/>
-      <c r="B16" s="3" t="s">
+      <c r="A16" s="5"/>
+      <c r="B16" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7">
+      <c r="C16" s="32"/>
+      <c r="D16" s="32">
         <v>285000</v>
       </c>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7">
+      <c r="E16" s="32"/>
+      <c r="F16" s="32"/>
+      <c r="G16" s="32">
         <f>SUM(C16:F16)</f>
         <v>285000</v>
       </c>
-      <c r="H16" s="2">
+      <c r="H16" s="6">
         <f>G16/$G$23</f>
         <v>2.925999020765661E-2</v>
       </c>
-      <c r="I16" s="2"/>
-      <c r="J16" s="1"/>
-      <c r="K16" s="1"/>
-      <c r="L16" s="1"/>
-      <c r="M16" s="1"/>
-      <c r="N16" s="1"/>
-      <c r="O16" s="1"/>
+      <c r="I16" s="6"/>
+      <c r="J16" s="5"/>
+      <c r="K16" s="5"/>
+      <c r="L16" s="5"/>
+      <c r="M16" s="5"/>
+      <c r="N16" s="5"/>
+      <c r="O16" s="5"/>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A17" s="1"/>
-      <c r="B17" s="3" t="s">
+      <c r="A17" s="5"/>
+      <c r="B17" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7">
+      <c r="C17" s="32"/>
+      <c r="D17" s="32"/>
+      <c r="E17" s="32">
         <v>96186</v>
       </c>
-      <c r="F17" s="7"/>
-      <c r="G17" s="7">
+      <c r="F17" s="32"/>
+      <c r="G17" s="32">
         <f>SUM(C17:F17)</f>
         <v>96186</v>
       </c>
-      <c r="H17" s="2">
+      <c r="H17" s="6">
         <f>G17/$G$23</f>
         <v>9.8750926951356455E-3</v>
       </c>
-      <c r="I17" s="2"/>
-      <c r="J17" s="1"/>
-      <c r="K17" s="1"/>
-      <c r="L17" s="1"/>
-      <c r="M17" s="1"/>
-      <c r="N17" s="1"/>
-      <c r="O17" s="1"/>
+      <c r="I17" s="6"/>
+      <c r="J17" s="5"/>
+      <c r="K17" s="5"/>
+      <c r="L17" s="5"/>
+      <c r="M17" s="5"/>
+      <c r="N17" s="5"/>
+      <c r="O17" s="5"/>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A18" s="1"/>
-      <c r="B18" s="3" t="s">
+      <c r="A18" s="5"/>
+      <c r="B18" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7">
+      <c r="C18" s="32"/>
+      <c r="D18" s="32"/>
+      <c r="E18" s="32">
         <v>48095</v>
       </c>
-      <c r="F18" s="7"/>
-      <c r="G18" s="7">
+      <c r="F18" s="32"/>
+      <c r="G18" s="32">
         <f>SUM(C18:F18)</f>
         <v>48095</v>
       </c>
-      <c r="H18" s="2">
+      <c r="H18" s="6">
         <f>G18/$G$23</f>
         <v>4.9377516808324371E-3</v>
       </c>
-      <c r="I18" s="2"/>
-      <c r="J18" s="1"/>
-      <c r="K18" s="1"/>
-      <c r="L18" s="1"/>
-      <c r="M18" s="1"/>
-      <c r="N18" s="1"/>
-      <c r="O18" s="1"/>
+      <c r="I18" s="6"/>
+      <c r="J18" s="5"/>
+      <c r="K18" s="5"/>
+      <c r="L18" s="5"/>
+      <c r="M18" s="5"/>
+      <c r="N18" s="5"/>
+      <c r="O18" s="5"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A19" s="1"/>
-      <c r="B19" s="3" t="s">
+      <c r="A19" s="5"/>
+      <c r="B19" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="7">
+      <c r="C19" s="32"/>
+      <c r="D19" s="32"/>
+      <c r="E19" s="32"/>
+      <c r="F19" s="32">
         <v>12395</v>
       </c>
-      <c r="G19" s="7">
+      <c r="G19" s="32">
         <f>SUM(C19:F19)</f>
         <v>12395</v>
       </c>
-      <c r="H19" s="2">
+      <c r="H19" s="6">
         <f>G19/$G$23</f>
         <v>1.2725529074522936E-3</v>
       </c>
-      <c r="I19" s="2"/>
-      <c r="J19" s="1"/>
-      <c r="K19" s="1"/>
-      <c r="L19" s="1"/>
-      <c r="M19" s="1"/>
-      <c r="N19" s="1"/>
-      <c r="O19" s="1"/>
+      <c r="I19" s="6"/>
+      <c r="J19" s="5"/>
+      <c r="K19" s="5"/>
+      <c r="L19" s="5"/>
+      <c r="M19" s="5"/>
+      <c r="N19" s="5"/>
+      <c r="O19" s="5"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A20" s="1"/>
-      <c r="B20" s="3" t="s">
+      <c r="A20" s="5"/>
+      <c r="B20" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="7">
+      <c r="C20" s="32"/>
+      <c r="D20" s="32"/>
+      <c r="E20" s="32"/>
+      <c r="F20" s="32">
         <v>8333</v>
       </c>
-      <c r="G20" s="7">
+      <c r="G20" s="32">
         <f>SUM(C20:F20)</f>
         <v>8333</v>
       </c>
-      <c r="H20" s="2">
+      <c r="H20" s="6">
         <f>G20/$G$23</f>
         <v>8.5552104701895626E-4</v>
       </c>
-      <c r="I20" s="2"/>
-      <c r="J20" s="1"/>
-      <c r="K20" s="1"/>
-      <c r="L20" s="1"/>
-      <c r="M20" s="1"/>
-      <c r="N20" s="1"/>
-      <c r="O20" s="1"/>
+      <c r="I20" s="6"/>
+      <c r="J20" s="5"/>
+      <c r="K20" s="5"/>
+      <c r="L20" s="5"/>
+      <c r="M20" s="5"/>
+      <c r="N20" s="5"/>
+      <c r="O20" s="5"/>
     </row>
     <row r="21" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="1"/>
-      <c r="B21" s="3" t="s">
+      <c r="A21" s="5"/>
+      <c r="B21" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7">
+      <c r="C21" s="32"/>
+      <c r="D21" s="32">
         <v>65105</v>
       </c>
-      <c r="E21" s="7"/>
-      <c r="F21" s="7"/>
-      <c r="G21" s="7">
+      <c r="E21" s="32"/>
+      <c r="F21" s="32"/>
+      <c r="G21" s="32">
         <f>SUM(C21:F21)</f>
         <v>65105</v>
       </c>
-      <c r="H21" s="2">
+      <c r="H21" s="6">
         <f>G21/$G$23</f>
         <v>6.6841110963841528E-3</v>
       </c>
-      <c r="I21" s="2"/>
-      <c r="J21" s="1"/>
-      <c r="K21" s="1"/>
-      <c r="L21" s="1"/>
-      <c r="M21" s="1"/>
-      <c r="N21" s="1"/>
-      <c r="O21" s="1"/>
+      <c r="I21" s="6"/>
+      <c r="J21" s="5"/>
+      <c r="K21" s="5"/>
+      <c r="L21" s="5"/>
+      <c r="M21" s="5"/>
+      <c r="N21" s="5"/>
+      <c r="O21" s="5"/>
     </row>
     <row r="22" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
-      <c r="H22" s="1"/>
-      <c r="I22" s="2"/>
-      <c r="J22" s="1"/>
-      <c r="K22" s="1"/>
-      <c r="L22" s="1"/>
-      <c r="M22" s="1"/>
-      <c r="N22" s="1"/>
-      <c r="O22" s="1"/>
+      <c r="A22" s="5"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="5"/>
+      <c r="I22" s="6"/>
+      <c r="J22" s="5"/>
+      <c r="K22" s="5"/>
+      <c r="L22" s="5"/>
+      <c r="M22" s="5"/>
+      <c r="N22" s="5"/>
+      <c r="O22" s="5"/>
     </row>
     <row r="23" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="1"/>
-      <c r="B23" s="4" t="s">
+      <c r="A23" s="5"/>
+      <c r="B23" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="C23" s="9">
+      <c r="C23" s="34">
         <f>SUM(C4:C21)</f>
         <v>8629687</v>
       </c>
-      <c r="D23" s="9">
+      <c r="D23" s="34">
         <f>SUM(D4:D21)</f>
         <v>879005</v>
       </c>
-      <c r="E23" s="9">
+      <c r="E23" s="34">
         <f>SUM(E4:E21)</f>
         <v>210843</v>
       </c>
-      <c r="F23" s="9">
+      <c r="F23" s="34">
         <f>SUM(F4:F21)</f>
         <v>20728</v>
       </c>
-      <c r="G23" s="9">
+      <c r="G23" s="34">
         <f>SUM(G4:G21)</f>
         <v>9740263</v>
       </c>
-      <c r="H23" s="7"/>
-      <c r="I23" s="7"/>
-      <c r="J23" s="1"/>
-      <c r="K23" s="1"/>
-      <c r="L23" s="1"/>
-      <c r="M23" s="1"/>
-      <c r="N23" s="1"/>
-      <c r="O23" s="1"/>
+      <c r="H23" s="32"/>
+      <c r="I23" s="32"/>
+      <c r="J23" s="5"/>
+      <c r="K23" s="5"/>
+      <c r="L23" s="5"/>
+      <c r="M23" s="5"/>
+      <c r="N23" s="5"/>
+      <c r="O23" s="5"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1780,148 +2147,796 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A1" s="5"/>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="5"/>
+      <c r="J1" s="5"/>
+      <c r="K1" s="5"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A2" s="5"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="33" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="5"/>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A3" s="5"/>
+      <c r="B3" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="5"/>
+      <c r="E3" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A4" s="5"/>
+      <c r="B4" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="18">
+        <v>25000</v>
+      </c>
+      <c r="D4" s="5"/>
+      <c r="E4" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
+      <c r="J4" s="5"/>
+      <c r="K4" s="5"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A5" s="5"/>
+      <c r="B5" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="18">
+        <v>25000</v>
+      </c>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
+      <c r="I5" s="5"/>
+      <c r="J5" s="5"/>
+      <c r="K5" s="5"/>
+    </row>
+    <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="5"/>
+      <c r="B6" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" s="18">
+        <v>137170.75</v>
+      </c>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
+      <c r="J6" s="5"/>
+      <c r="K6" s="5"/>
+    </row>
+    <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="5"/>
+      <c r="B7" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="18">
+        <v>3846829.25</v>
+      </c>
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
+      <c r="I7" s="5"/>
+      <c r="J7" s="5"/>
+      <c r="K7" s="5"/>
+    </row>
+    <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="5"/>
+      <c r="B8" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="18">
+        <v>16566</v>
+      </c>
+      <c r="D8" s="5"/>
+      <c r="E8" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
+      <c r="I8" s="5"/>
+      <c r="J8" s="5"/>
+      <c r="K8" s="5"/>
+    </row>
+    <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="5"/>
+      <c r="B9" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="18">
+        <v>250000</v>
+      </c>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="5"/>
+      <c r="J9" s="5"/>
+      <c r="K9" s="5"/>
+    </row>
+    <row r="10" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="5"/>
+      <c r="B10" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" s="18">
+        <v>100000</v>
+      </c>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="5"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5"/>
+      <c r="J10" s="5"/>
+      <c r="K10" s="5"/>
+    </row>
+    <row r="11" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="5"/>
+      <c r="B11" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" s="18">
+        <v>300000</v>
+      </c>
+      <c r="D11" s="5"/>
+      <c r="E11" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="5"/>
+      <c r="I11" s="5"/>
+      <c r="J11" s="5"/>
+      <c r="K11" s="5"/>
+    </row>
+    <row r="12" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="5"/>
+      <c r="B12" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="18">
+        <v>37500</v>
+      </c>
+      <c r="D12" s="5"/>
+      <c r="E12" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="F12" s="5"/>
+      <c r="G12" s="5"/>
+      <c r="H12" s="5"/>
+      <c r="I12" s="5"/>
+      <c r="J12" s="5"/>
+      <c r="K12" s="5"/>
+    </row>
+    <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="5"/>
+      <c r="B13" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="C13" s="18">
+        <v>250000</v>
+      </c>
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="5"/>
+      <c r="H13" s="5"/>
+      <c r="I13" s="5"/>
+      <c r="J13" s="5"/>
+      <c r="K13" s="5"/>
+    </row>
+    <row r="14" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="5"/>
+      <c r="B14" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" s="18">
+        <v>100000</v>
+      </c>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
+      <c r="I14" s="5"/>
+      <c r="J14" s="5"/>
+      <c r="K14" s="5"/>
+    </row>
+    <row r="15" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="5"/>
+      <c r="B15" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="C15" s="18">
+        <v>41164</v>
+      </c>
+      <c r="D15" s="5"/>
+      <c r="E15" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="F15" s="5"/>
+      <c r="G15" s="5"/>
+      <c r="H15" s="5"/>
+      <c r="I15" s="5"/>
+      <c r="J15" s="5"/>
+      <c r="K15" s="5"/>
+    </row>
+    <row r="16" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="5"/>
+      <c r="B16" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="C16" s="18">
+        <v>2328778</v>
+      </c>
+      <c r="D16" s="5"/>
+      <c r="E16" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="F16" s="5"/>
+      <c r="G16" s="5"/>
+      <c r="H16" s="5"/>
+      <c r="I16" s="5"/>
+      <c r="J16" s="5"/>
+      <c r="K16" s="5"/>
+    </row>
+    <row r="17" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="5"/>
+      <c r="B17" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="C17" s="18">
+        <v>1506000</v>
+      </c>
+      <c r="D17" s="5"/>
+      <c r="E17" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="F17" s="5"/>
+      <c r="G17" s="5"/>
+      <c r="H17" s="5"/>
+      <c r="I17" s="5"/>
+      <c r="J17" s="5"/>
+      <c r="K17" s="5"/>
+    </row>
+    <row r="18" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="5"/>
+      <c r="B18" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="C18" s="18">
+        <v>50000</v>
+      </c>
+      <c r="D18" s="5"/>
+      <c r="E18" s="5"/>
+      <c r="F18" s="5"/>
+      <c r="G18" s="5"/>
+      <c r="H18" s="5"/>
+      <c r="I18" s="5"/>
+      <c r="J18" s="5"/>
+      <c r="K18" s="5"/>
+    </row>
+    <row r="19" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="5"/>
+      <c r="B19" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="C19" s="18">
+        <v>212500</v>
+      </c>
+      <c r="D19" s="5"/>
+      <c r="E19" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="F19" s="5"/>
+      <c r="G19" s="5"/>
+      <c r="H19" s="5"/>
+      <c r="I19" s="5"/>
+      <c r="J19" s="5"/>
+      <c r="K19" s="5"/>
+    </row>
+    <row r="20" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="5"/>
+      <c r="B20" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20" s="18">
+        <v>25000</v>
+      </c>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="5"/>
+      <c r="H20" s="5"/>
+      <c r="I20" s="5"/>
+      <c r="J20" s="5"/>
+      <c r="K20" s="5"/>
+    </row>
+    <row r="21" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="5"/>
+      <c r="B21" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="C21" s="18">
+        <v>61746</v>
+      </c>
+      <c r="D21" s="5"/>
+      <c r="E21" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="F21" s="5"/>
+      <c r="G21" s="5"/>
+      <c r="H21" s="5"/>
+      <c r="I21" s="5"/>
+      <c r="J21" s="5"/>
+      <c r="K21" s="5"/>
+    </row>
+    <row r="22" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="5"/>
+      <c r="B22" s="15" t="s">
+        <v>47</v>
+      </c>
+      <c r="C22" s="18">
+        <v>100000</v>
+      </c>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+      <c r="G22" s="5"/>
+      <c r="H22" s="5"/>
+      <c r="I22" s="5"/>
+      <c r="J22" s="5"/>
+      <c r="K22" s="5"/>
+    </row>
+    <row r="23" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="5"/>
+      <c r="B23" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="C23" s="18">
+        <v>100000</v>
+      </c>
+      <c r="D23" s="5"/>
+      <c r="E23" s="5"/>
+      <c r="F23" s="5"/>
+      <c r="G23" s="5"/>
+      <c r="H23" s="5"/>
+      <c r="I23" s="5"/>
+      <c r="J23" s="5"/>
+      <c r="K23" s="5"/>
+    </row>
+    <row r="24" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="5"/>
+      <c r="B24" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="C24" s="18">
+        <v>61746</v>
+      </c>
+      <c r="D24" s="5"/>
+      <c r="E24" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="F24" s="5"/>
+      <c r="G24" s="5"/>
+      <c r="H24" s="5"/>
+      <c r="I24" s="5"/>
+      <c r="J24" s="5"/>
+      <c r="K24" s="5"/>
+    </row>
+    <row r="25" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="5"/>
+      <c r="B25" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="C25" s="18">
+        <v>250000</v>
+      </c>
+      <c r="D25" s="5"/>
+      <c r="E25" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="F25" s="5"/>
+      <c r="G25" s="5"/>
+      <c r="H25" s="5"/>
+      <c r="I25" s="5"/>
+      <c r="J25" s="5"/>
+      <c r="K25" s="5"/>
+    </row>
+    <row r="26" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="5"/>
+      <c r="B26" s="5"/>
+      <c r="C26" s="33"/>
+      <c r="D26" s="5"/>
+      <c r="E26" s="5"/>
+      <c r="F26" s="5"/>
+      <c r="G26" s="5"/>
+      <c r="H26" s="5"/>
+      <c r="I26" s="5"/>
+      <c r="J26" s="5"/>
+      <c r="K26" s="5"/>
+    </row>
+    <row r="27" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="5"/>
+      <c r="B27" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="C27" s="17">
+        <f>SUM(C4:C25)</f>
+        <v>9825000</v>
+      </c>
+      <c r="D27" s="5"/>
+      <c r="E27" s="5"/>
+      <c r="F27" s="5"/>
+      <c r="G27" s="5"/>
+      <c r="H27" s="5"/>
+      <c r="I27" s="5"/>
+      <c r="J27" s="5"/>
+      <c r="K27" s="5"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C939BD08-A3E7-914E-B2D5-667E37178D18}">
+  <dimension ref="A1:X33"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="6.33203125" customWidth="1"/>
+    <col min="2" max="2" width="35.5" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="17.6640625" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="0.5" customWidth="1"/>
+    <col min="7" max="7" width="13.83203125" customWidth="1"/>
+    <col min="8" max="8" width="0.5" customWidth="1"/>
+    <col min="9" max="9" width="15.5" customWidth="1"/>
+    <col min="10" max="10" width="16.83203125" customWidth="1"/>
+    <col min="11" max="11" width="0.5" customWidth="1"/>
+    <col min="12" max="12" width="13.83203125" customWidth="1"/>
+    <col min="13" max="13" width="0.5" customWidth="1"/>
+    <col min="14" max="14" width="15.5" customWidth="1"/>
+    <col min="15" max="15" width="16.83203125" customWidth="1"/>
+    <col min="16" max="16" width="0.5" customWidth="1"/>
+    <col min="17" max="17" width="13.83203125" customWidth="1"/>
+    <col min="18" max="18" width="0.5" customWidth="1"/>
+    <col min="19" max="19" width="15.5" customWidth="1"/>
+    <col min="20" max="20" width="9.33203125" customWidth="1"/>
+    <col min="21" max="21" width="6.83203125" customWidth="1"/>
+    <col min="22" max="22" width="15.5" customWidth="1"/>
+    <col min="23" max="23" width="13" customWidth="1"/>
+    <col min="24" max="24" width="10.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A1" s="1"/>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="B1" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="7"/>
+      <c r="L1" s="7"/>
+      <c r="M1" s="7"/>
+      <c r="N1" s="7"/>
+      <c r="O1" s="7"/>
+      <c r="P1" s="7"/>
+      <c r="Q1" s="7"/>
+      <c r="R1" s="7"/>
+      <c r="S1" s="7"/>
+      <c r="T1" s="7"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="1"/>
+      <c r="W1" s="1"/>
+      <c r="X1" s="1"/>
+    </row>
+    <row r="2" spans="1:24" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="8" t="s">
+      <c r="B2" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="7"/>
+      <c r="K2" s="7"/>
+      <c r="L2" s="7"/>
+      <c r="M2" s="7"/>
+      <c r="N2" s="7"/>
+      <c r="O2" s="7"/>
+      <c r="P2" s="7"/>
+      <c r="Q2" s="7"/>
+      <c r="R2" s="7"/>
+      <c r="S2" s="7"/>
+      <c r="T2" s="7"/>
+      <c r="U2" s="1"/>
+      <c r="V2" s="1"/>
+      <c r="W2" s="1"/>
+      <c r="X2" s="1"/>
+    </row>
+    <row r="3" spans="1:24" ht="16.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="1"/>
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+      <c r="K3" s="4"/>
+      <c r="L3" s="4"/>
+      <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
+      <c r="P3" s="4"/>
+      <c r="Q3" s="4"/>
+      <c r="R3" s="4"/>
+      <c r="S3" s="4"/>
+      <c r="T3" s="4"/>
+      <c r="U3" s="1"/>
+      <c r="V3" s="1"/>
+      <c r="W3" s="1"/>
+      <c r="X3" s="1"/>
+    </row>
+    <row r="4" spans="1:24" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="1"/>
+      <c r="B4" s="1"/>
+      <c r="C4" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="D4" s="40" t="s">
         <v>26</v>
       </c>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" s="1"/>
-      <c r="B3" s="4" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D3" s="1"/>
-      <c r="E3" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" s="1"/>
-      <c r="B4" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="6">
-        <v>25000</v>
-      </c>
-      <c r="D4" s="1"/>
-      <c r="E4" s="3" t="s">
-        <v>28</v>
-      </c>
+      <c r="E4" s="41"/>
       <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
+      <c r="G4" s="27" t="s">
+        <v>54</v>
+      </c>
       <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
+      <c r="I4" s="40" t="s">
+        <v>55</v>
+      </c>
+      <c r="J4" s="41"/>
       <c r="K4" s="1"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="L4" s="27" t="s">
+        <v>54</v>
+      </c>
+      <c r="M4" s="1"/>
+      <c r="N4" s="40" t="s">
+        <v>56</v>
+      </c>
+      <c r="O4" s="41"/>
+      <c r="P4" s="1"/>
+      <c r="Q4" s="1"/>
+      <c r="R4" s="1"/>
+      <c r="S4" s="1"/>
+      <c r="T4" s="1"/>
+      <c r="U4" s="1"/>
+      <c r="V4" s="1"/>
+      <c r="W4" s="1"/>
+      <c r="X4" s="1"/>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A5" s="1"/>
-      <c r="B5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" s="6">
-        <v>25000</v>
-      </c>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
-      <c r="K5" s="1"/>
-    </row>
-    <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B5" s="1"/>
+      <c r="C5" s="22" t="s">
+        <v>57</v>
+      </c>
+      <c r="D5" s="22" t="s">
+        <v>58</v>
+      </c>
+      <c r="E5" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="F5" s="20"/>
+      <c r="G5" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="H5" s="20"/>
+      <c r="I5" s="22" t="s">
+        <v>58</v>
+      </c>
+      <c r="J5" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="K5" s="20"/>
+      <c r="L5" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="M5" s="20"/>
+      <c r="N5" s="22" t="s">
+        <v>61</v>
+      </c>
+      <c r="O5" s="23" t="s">
+        <v>84</v>
+      </c>
+      <c r="P5" s="1"/>
+      <c r="Q5" s="1"/>
+      <c r="R5" s="1"/>
+      <c r="S5" s="1"/>
+      <c r="T5" s="1"/>
+      <c r="U5" s="1"/>
+      <c r="V5" s="1"/>
+      <c r="W5" s="1"/>
+      <c r="X5" s="1"/>
+    </row>
+    <row r="6" spans="1:24" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
-      <c r="B6" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C6" s="6">
-        <v>137170.75</v>
-      </c>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
-    </row>
-    <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B6" s="1"/>
+      <c r="C6" s="24" t="s">
+        <v>62</v>
+      </c>
+      <c r="D6" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="E6" s="25" t="s">
+        <v>62</v>
+      </c>
+      <c r="F6" s="20"/>
+      <c r="G6" s="28" t="s">
+        <v>77</v>
+      </c>
+      <c r="H6" s="20"/>
+      <c r="I6" s="24" t="s">
+        <v>63</v>
+      </c>
+      <c r="J6" s="25" t="s">
+        <v>62</v>
+      </c>
+      <c r="K6" s="20"/>
+      <c r="L6" s="28" t="s">
+        <v>64</v>
+      </c>
+      <c r="M6" s="20"/>
+      <c r="N6" s="24" t="s">
+        <v>62</v>
+      </c>
+      <c r="O6" s="21" t="s">
+        <v>65</v>
+      </c>
+      <c r="P6" s="1"/>
+      <c r="Q6" s="1"/>
+      <c r="R6" s="1"/>
+      <c r="S6" s="1"/>
+      <c r="T6" s="1"/>
+      <c r="U6" s="1"/>
+      <c r="V6" s="1"/>
+      <c r="W6" s="1"/>
+      <c r="X6" s="1"/>
+    </row>
+    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A7" s="1"/>
-      <c r="B7" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C7" s="6">
-        <v>3846829.25</v>
-      </c>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
-      <c r="K7" s="1"/>
-    </row>
-    <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B7" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="C7" s="39"/>
+      <c r="D7" s="39"/>
+      <c r="E7" s="39"/>
+      <c r="F7" s="14"/>
+      <c r="G7" s="39"/>
+      <c r="H7" s="14"/>
+      <c r="I7" s="39"/>
+      <c r="J7" s="39"/>
+      <c r="K7" s="14"/>
+      <c r="L7" s="39"/>
+      <c r="M7" s="14"/>
+      <c r="N7" s="39"/>
+      <c r="O7" s="42"/>
+      <c r="P7" s="1"/>
+      <c r="Q7" s="1"/>
+      <c r="R7" s="1"/>
+      <c r="S7" s="1"/>
+      <c r="T7" s="1"/>
+      <c r="U7" s="1"/>
+      <c r="V7" s="1"/>
+      <c r="W7" s="1"/>
+      <c r="X7" s="1"/>
+    </row>
+    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A8" s="1"/>
-      <c r="B8" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C8" s="6">
-        <v>16566</v>
+      <c r="B8" s="30" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="11">
+        <f>DetailedCapTable!G4</f>
+        <v>3600000</v>
       </c>
       <c r="D8" s="1"/>
-      <c r="E8" s="3" t="s">
-        <v>52</v>
-      </c>
+      <c r="E8" s="1"/>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
-    </row>
-    <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
+      <c r="N8" s="12">
+        <f>C8</f>
+        <v>3600000</v>
+      </c>
+      <c r="O8" s="43">
+        <f ca="1">N8/$N$21</f>
+        <v>0.18702018607573415</v>
+      </c>
+      <c r="P8" s="1"/>
+      <c r="Q8" s="1"/>
+      <c r="R8" s="1"/>
+      <c r="S8" s="1"/>
+      <c r="T8" s="1"/>
+      <c r="U8" s="1"/>
+      <c r="V8" s="1"/>
+      <c r="W8" s="1"/>
+      <c r="X8" s="1"/>
+    </row>
+    <row r="9" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A9" s="1"/>
-      <c r="B9" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" s="6">
-        <v>250000</v>
+      <c r="B9" s="30" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="11">
+        <f>DetailedCapTable!G5</f>
+        <v>3600000</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
@@ -1931,14 +2946,34 @@
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
-    </row>
-    <row r="10" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L9" s="1"/>
+      <c r="M9" s="1"/>
+      <c r="N9" s="12">
+        <f>C9</f>
+        <v>3600000</v>
+      </c>
+      <c r="O9" s="43">
+        <f ca="1">N9/$N$21</f>
+        <v>0.18702018607573415</v>
+      </c>
+      <c r="P9" s="1"/>
+      <c r="Q9" s="1"/>
+      <c r="R9" s="1"/>
+      <c r="S9" s="1"/>
+      <c r="T9" s="1"/>
+      <c r="U9" s="1"/>
+      <c r="V9" s="1"/>
+      <c r="W9" s="1"/>
+      <c r="X9" s="1"/>
+    </row>
+    <row r="10" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A10" s="1"/>
-      <c r="B10" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C10" s="6">
-        <v>100000</v>
+      <c r="B10" s="30" t="s">
+        <v>78</v>
+      </c>
+      <c r="C10" s="11">
+        <f>SUM(DetailedCapTable!G6:'DetailedCapTable'!G20)</f>
+        <v>2475158</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
@@ -1948,53 +2983,115 @@
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
-    </row>
-    <row r="11" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L10" s="1"/>
+      <c r="M10" s="1"/>
+      <c r="N10" s="12">
+        <f>C10</f>
+        <v>2475158</v>
+      </c>
+      <c r="O10" s="43">
+        <f ca="1">N10/$N$21</f>
+        <v>0.12858458603523387</v>
+      </c>
+      <c r="P10" s="1"/>
+      <c r="Q10" s="1"/>
+      <c r="R10" s="1"/>
+      <c r="S10" s="1"/>
+      <c r="T10" s="1"/>
+      <c r="U10" s="1"/>
+      <c r="V10" s="1"/>
+      <c r="W10" s="1"/>
+      <c r="X10" s="1"/>
+    </row>
+    <row r="11" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A11" s="1"/>
-      <c r="B11" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="C11" s="6">
-        <v>300000</v>
-      </c>
+      <c r="B11" s="30" t="s">
+        <v>79</v>
+      </c>
+      <c r="C11" s="1"/>
       <c r="D11" s="1"/>
-      <c r="E11" s="3" t="s">
-        <v>28</v>
-      </c>
+      <c r="E11" s="1"/>
       <c r="F11" s="1"/>
-      <c r="G11" s="1"/>
+      <c r="G11" s="11">
+        <f>DetailedCapTable!G21</f>
+        <v>65105</v>
+      </c>
       <c r="H11" s="1"/>
       <c r="I11" s="1"/>
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
-    </row>
-    <row r="12" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L11" s="12">
+        <f ca="1">ROUND(0.1*N21-G11,0)</f>
+        <v>1859821</v>
+      </c>
+      <c r="M11" s="1"/>
+      <c r="N11" s="12">
+        <f ca="1">G11+L11</f>
+        <v>1924926</v>
+      </c>
+      <c r="O11" s="43">
+        <f ca="1">N11/$N$21</f>
+        <v>0.10000000519500517</v>
+      </c>
+      <c r="P11" s="1"/>
+      <c r="Q11" s="1"/>
+      <c r="R11" s="1"/>
+      <c r="S11" s="1"/>
+      <c r="T11" s="1"/>
+      <c r="U11" s="1"/>
+      <c r="V11" s="1"/>
+      <c r="W11" s="1"/>
+      <c r="X11" s="1"/>
+    </row>
+    <row r="12" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A12" s="1"/>
-      <c r="B12" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="C12" s="6">
-        <v>37500</v>
+      <c r="B12" s="31" t="s">
+        <v>67</v>
+      </c>
+      <c r="C12" s="46">
+        <f>SUM(C8:C11)</f>
+        <v>9675158</v>
       </c>
       <c r="D12" s="1"/>
-      <c r="E12" s="3" t="s">
-        <v>36</v>
-      </c>
+      <c r="E12" s="1"/>
       <c r="F12" s="1"/>
-      <c r="G12" s="1"/>
+      <c r="G12" s="46">
+        <f>G11</f>
+        <v>65105</v>
+      </c>
       <c r="H12" s="1"/>
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
-    </row>
-    <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L12" s="46">
+        <f ca="1">L11</f>
+        <v>1859821</v>
+      </c>
+      <c r="M12" s="1"/>
+      <c r="N12" s="12">
+        <f ca="1">SUM(N8:N11)</f>
+        <v>11600084</v>
+      </c>
+      <c r="O12" s="43">
+        <f ca="1">N12/$N$21</f>
+        <v>0.60262496338170735</v>
+      </c>
+      <c r="P12" s="1"/>
+      <c r="Q12" s="1"/>
+      <c r="R12" s="1"/>
+      <c r="S12" s="1"/>
+      <c r="T12" s="1"/>
+      <c r="U12" s="1"/>
+      <c r="V12" s="1"/>
+      <c r="W12" s="1"/>
+      <c r="X12" s="1"/>
+    </row>
+    <row r="13" spans="1:24" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="1"/>
-      <c r="B13" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C13" s="6">
-        <v>250000</v>
-      </c>
+      <c r="B13" s="31" t="s">
+        <v>68</v>
+      </c>
+      <c r="C13" s="1"/>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
@@ -2003,35 +3100,76 @@
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
       <c r="K13" s="1"/>
-    </row>
-    <row r="14" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L13" s="1"/>
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
+      <c r="O13" s="44"/>
+      <c r="P13" s="1"/>
+      <c r="Q13" s="1"/>
+      <c r="R13" s="1"/>
+      <c r="S13" s="1"/>
+      <c r="T13" s="1"/>
+      <c r="U13" s="1"/>
+      <c r="V13" s="1"/>
+      <c r="W13" s="1"/>
+      <c r="X13" s="1"/>
+    </row>
+    <row r="14" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A14" s="1"/>
-      <c r="B14" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C14" s="6">
-        <v>100000</v>
-      </c>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
+      <c r="B14" s="30" t="s">
+        <v>42</v>
+      </c>
+      <c r="C14" s="1"/>
+      <c r="D14" s="35">
+        <v>8000000</v>
+      </c>
+      <c r="E14" s="11">
+        <f ca="1">IFERROR(ROUND(D14/E23,0),0)</f>
+        <v>2309911</v>
+      </c>
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
       <c r="H14" s="1"/>
-      <c r="I14" s="1"/>
-      <c r="J14" s="1"/>
+      <c r="I14" s="35">
+        <v>5000000</v>
+      </c>
+      <c r="J14" s="12">
+        <f ca="1">IFERROR(ROUND(I14/J23,0),0)</f>
+        <v>1203079</v>
+      </c>
       <c r="K14" s="1"/>
-    </row>
-    <row r="15" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L14" s="1"/>
+      <c r="M14" s="1"/>
+      <c r="N14" s="12">
+        <f ca="1">E14+J14</f>
+        <v>3512990</v>
+      </c>
+      <c r="O14" s="43">
+        <f ca="1">N14/$N$21</f>
+        <v>0.18250001207838701</v>
+      </c>
+      <c r="P14" s="1"/>
+      <c r="Q14" s="1"/>
+      <c r="R14" s="1"/>
+      <c r="S14" s="1"/>
+      <c r="T14" s="1"/>
+      <c r="U14" s="1"/>
+      <c r="V14" s="1"/>
+      <c r="W14" s="1"/>
+      <c r="X14" s="1"/>
+    </row>
+    <row r="15" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A15" s="1"/>
-      <c r="B15" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C15" s="6">
-        <v>41164</v>
-      </c>
-      <c r="D15" s="1"/>
-      <c r="E15" s="3" t="s">
-        <v>52</v>
+      <c r="B15" s="30" t="s">
+        <v>69</v>
+      </c>
+      <c r="C15" s="1"/>
+      <c r="D15" s="35">
+        <v>250000</v>
+      </c>
+      <c r="E15" s="12">
+        <f ca="1">IFERROR(ROUND(D15/E23,0),0)</f>
+        <v>72185</v>
       </c>
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
@@ -2039,18 +3177,38 @@
       <c r="I15" s="1"/>
       <c r="J15" s="1"/>
       <c r="K15" s="1"/>
-    </row>
-    <row r="16" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L15" s="1"/>
+      <c r="M15" s="1"/>
+      <c r="N15" s="12">
+        <f ca="1">E15+J15</f>
+        <v>72185</v>
+      </c>
+      <c r="O15" s="43">
+        <f ca="1">N15/$N$21</f>
+        <v>3.7500144810769078E-3</v>
+      </c>
+      <c r="P15" s="1"/>
+      <c r="Q15" s="1"/>
+      <c r="R15" s="1"/>
+      <c r="S15" s="1"/>
+      <c r="T15" s="1"/>
+      <c r="U15" s="1"/>
+      <c r="V15" s="1"/>
+      <c r="W15" s="1"/>
+      <c r="X15" s="1"/>
+    </row>
+    <row r="16" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A16" s="1"/>
-      <c r="B16" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C16" s="6">
-        <v>2328778</v>
-      </c>
-      <c r="D16" s="1"/>
-      <c r="E16" s="3" t="s">
-        <v>52</v>
+      <c r="B16" s="30" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16" s="1"/>
+      <c r="D16" s="35">
+        <v>300000</v>
+      </c>
+      <c r="E16" s="12">
+        <f ca="1">IFERROR(ROUND(D16/E23,0),0)</f>
+        <v>86622</v>
       </c>
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
@@ -2058,18 +3216,38 @@
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
       <c r="K16" s="1"/>
-    </row>
-    <row r="17" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L16" s="1"/>
+      <c r="M16" s="1"/>
+      <c r="N16" s="12">
+        <f ca="1">E16+J16</f>
+        <v>86622</v>
+      </c>
+      <c r="O16" s="43">
+        <f ca="1">N16/$N$21</f>
+        <v>4.5000173772922897E-3</v>
+      </c>
+      <c r="P16" s="1"/>
+      <c r="Q16" s="1"/>
+      <c r="R16" s="1"/>
+      <c r="S16" s="1"/>
+      <c r="T16" s="1"/>
+      <c r="U16" s="1"/>
+      <c r="V16" s="1"/>
+      <c r="W16" s="1"/>
+      <c r="X16" s="1"/>
+    </row>
+    <row r="17" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A17" s="1"/>
-      <c r="B17" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="C17" s="6">
-        <v>1506000</v>
-      </c>
-      <c r="D17" s="1"/>
-      <c r="E17" s="3" t="s">
-        <v>42</v>
+      <c r="B17" s="30" t="s">
+        <v>80</v>
+      </c>
+      <c r="C17" s="1"/>
+      <c r="D17" s="35">
+        <v>1275000</v>
+      </c>
+      <c r="E17" s="12">
+        <f ca="1">IFERROR(ROUND(D17/E23,0),0)</f>
+        <v>368142</v>
       </c>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
@@ -2077,51 +3255,108 @@
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
       <c r="K17" s="1"/>
-    </row>
-    <row r="18" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L17" s="1"/>
+      <c r="M17" s="1"/>
+      <c r="N17" s="12">
+        <f ca="1">E17+J17</f>
+        <v>368142</v>
+      </c>
+      <c r="O17" s="43">
+        <f ca="1">N17/$N$21</f>
+        <v>1.9124995928414698E-2</v>
+      </c>
+      <c r="P17" s="1"/>
+      <c r="Q17" s="1"/>
+      <c r="R17" s="1"/>
+      <c r="S17" s="1"/>
+      <c r="T17" s="1"/>
+      <c r="U17" s="1"/>
+      <c r="V17" s="1"/>
+      <c r="W17" s="1"/>
+      <c r="X17" s="1"/>
+    </row>
+    <row r="18" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A18" s="1"/>
-      <c r="B18" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C18" s="6">
-        <v>50000</v>
-      </c>
+      <c r="B18" s="30" t="s">
+        <v>87</v>
+      </c>
+      <c r="C18" s="1"/>
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
-      <c r="J18" s="1"/>
+      <c r="I18" s="35">
+        <v>12000000</v>
+      </c>
+      <c r="J18" s="12">
+        <f ca="1">IFERROR(ROUND(I18/J23,0),0)</f>
+        <v>2887389</v>
+      </c>
       <c r="K18" s="1"/>
-    </row>
-    <row r="19" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L18" s="1"/>
+      <c r="M18" s="1"/>
+      <c r="N18" s="12">
+        <f ca="1">E18+J18</f>
+        <v>2887389</v>
+      </c>
+      <c r="O18" s="43">
+        <f ca="1">N18/$N$21</f>
+        <v>0.15000000779250774</v>
+      </c>
+      <c r="P18" s="1"/>
+      <c r="Q18" s="1"/>
+      <c r="R18" s="1"/>
+      <c r="S18" s="1"/>
+      <c r="T18" s="1"/>
+      <c r="U18" s="1"/>
+      <c r="V18" s="1"/>
+      <c r="W18" s="1"/>
+      <c r="X18" s="1"/>
+    </row>
+    <row r="19" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A19" s="1"/>
-      <c r="B19" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="C19" s="6">
-        <v>212500</v>
-      </c>
+      <c r="B19" s="30" t="s">
+        <v>81</v>
+      </c>
+      <c r="C19" s="1"/>
       <c r="D19" s="1"/>
-      <c r="E19" s="3" t="s">
-        <v>36</v>
-      </c>
+      <c r="E19" s="1"/>
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
-      <c r="I19" s="1"/>
-      <c r="J19" s="1"/>
+      <c r="I19" s="35">
+        <v>3000000</v>
+      </c>
+      <c r="J19" s="12">
+        <f ca="1">IFERROR(ROUND(I19/J23,0),0)</f>
+        <v>721847</v>
+      </c>
       <c r="K19" s="1"/>
-    </row>
-    <row r="20" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L19" s="1"/>
+      <c r="M19" s="1"/>
+      <c r="N19" s="12">
+        <f ca="1">E19+J19</f>
+        <v>721847</v>
+      </c>
+      <c r="O19" s="43">
+        <f ca="1">N19/$N$21</f>
+        <v>3.7499988960614017E-2</v>
+      </c>
+      <c r="P19" s="1"/>
+      <c r="Q19" s="1"/>
+      <c r="R19" s="1"/>
+      <c r="S19" s="1"/>
+      <c r="T19" s="1"/>
+      <c r="U19" s="1"/>
+      <c r="V19" s="1"/>
+      <c r="W19" s="1"/>
+      <c r="X19" s="1"/>
+    </row>
+    <row r="20" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A20" s="1"/>
-      <c r="B20" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="C20" s="6">
-        <v>25000</v>
-      </c>
+      <c r="B20" s="9"/>
+      <c r="C20" s="1"/>
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
@@ -2130,34 +3365,79 @@
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
       <c r="K20" s="1"/>
-    </row>
-    <row r="21" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L20" s="1"/>
+      <c r="M20" s="1"/>
+      <c r="N20" s="1"/>
+      <c r="O20" s="44"/>
+      <c r="P20" s="1"/>
+      <c r="Q20" s="1"/>
+      <c r="R20" s="1"/>
+      <c r="S20" s="1"/>
+      <c r="T20" s="1"/>
+      <c r="U20" s="1"/>
+      <c r="V20" s="1"/>
+      <c r="W20" s="1"/>
+      <c r="X20" s="1"/>
+    </row>
+    <row r="21" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A21" s="1"/>
-      <c r="B21" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C21" s="6">
-        <v>61746</v>
-      </c>
-      <c r="D21" s="1"/>
-      <c r="E21" s="3" t="s">
-        <v>52</v>
+      <c r="B21" s="31" t="s">
+        <v>70</v>
+      </c>
+      <c r="C21" s="46">
+        <f>C12</f>
+        <v>9675158</v>
+      </c>
+      <c r="D21" s="48">
+        <f>SUM(D14:D19)</f>
+        <v>9825000</v>
+      </c>
+      <c r="E21" s="47">
+        <f ca="1">SUM(E14:E19)</f>
+        <v>2836860</v>
       </c>
       <c r="F21" s="1"/>
-      <c r="G21" s="1"/>
+      <c r="G21" s="12">
+        <f>G11</f>
+        <v>65105</v>
+      </c>
       <c r="H21" s="1"/>
-      <c r="I21" s="1"/>
-      <c r="J21" s="1"/>
+      <c r="I21" s="48">
+        <f>SUM(I14:I19)</f>
+        <v>20000000</v>
+      </c>
+      <c r="J21" s="47">
+        <f ca="1">SUM(J14:J19)</f>
+        <v>4812315</v>
+      </c>
       <c r="K21" s="1"/>
-    </row>
-    <row r="22" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L21" s="12">
+        <f ca="1">L11</f>
+        <v>1859821</v>
+      </c>
+      <c r="M21" s="1"/>
+      <c r="N21" s="47">
+        <f ca="1">C12+G11+E21+L11+J21</f>
+        <v>19249259</v>
+      </c>
+      <c r="O21" s="49">
+        <f ca="1">N21/$N$21</f>
+        <v>1</v>
+      </c>
+      <c r="P21" s="1"/>
+      <c r="Q21" s="1"/>
+      <c r="R21" s="1"/>
+      <c r="S21" s="1"/>
+      <c r="T21" s="1"/>
+      <c r="U21" s="1"/>
+      <c r="V21" s="1"/>
+      <c r="W21" s="1"/>
+      <c r="X21" s="1"/>
+    </row>
+    <row r="22" spans="1:24" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="1"/>
-      <c r="B22" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="C22" s="6">
-        <v>100000</v>
-      </c>
+      <c r="B22" s="9"/>
+      <c r="C22" s="13"/>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
@@ -2166,66 +3446,124 @@
       <c r="I22" s="1"/>
       <c r="J22" s="1"/>
       <c r="K22" s="1"/>
-    </row>
-    <row r="23" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L22" s="1"/>
+      <c r="M22" s="1"/>
+      <c r="N22" s="1"/>
+      <c r="O22" s="44"/>
+      <c r="P22" s="1"/>
+      <c r="Q22" s="1"/>
+      <c r="R22" s="1"/>
+      <c r="S22" s="1"/>
+      <c r="T22" s="1"/>
+      <c r="U22" s="1"/>
+      <c r="V22" s="1"/>
+      <c r="W22" s="1"/>
+      <c r="X22" s="1"/>
+    </row>
+    <row r="23" spans="1:24" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="1"/>
-      <c r="B23" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="C23" s="6">
-        <v>100000</v>
-      </c>
+      <c r="B23" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="C23" s="1"/>
       <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
+      <c r="E23" s="36">
+        <f ca="1">IFERROR(50000000/(C12+G11+L11+E21),0)</f>
+        <v>3.4633368391537709</v>
+      </c>
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
-      <c r="J23" s="1"/>
+      <c r="J23" s="36">
+        <f ca="1">IFERROR(J24/(C12+G11+L11+E21),0)</f>
+        <v>4.1560042069845249</v>
+      </c>
       <c r="K23" s="1"/>
-    </row>
-    <row r="24" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L23" s="1"/>
+      <c r="M23" s="1"/>
+      <c r="N23" s="1"/>
+      <c r="O23" s="44"/>
+      <c r="P23" s="1"/>
+      <c r="Q23" s="1"/>
+      <c r="R23" s="1"/>
+      <c r="S23" s="1"/>
+      <c r="T23" s="1"/>
+      <c r="U23" s="1"/>
+      <c r="V23" s="1"/>
+      <c r="W23" s="1"/>
+      <c r="X23" s="1"/>
+    </row>
+    <row r="24" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A24" s="1"/>
-      <c r="B24" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="C24" s="6">
-        <v>61746</v>
-      </c>
+      <c r="B24" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C24" s="1"/>
       <c r="D24" s="1"/>
-      <c r="E24" s="3" t="s">
-        <v>52</v>
+      <c r="E24" s="35">
+        <v>50000000</v>
       </c>
       <c r="F24" s="1"/>
       <c r="G24" s="1"/>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
-      <c r="J24" s="1"/>
+      <c r="J24" s="35">
+        <v>60000000</v>
+      </c>
       <c r="K24" s="1"/>
-    </row>
-    <row r="25" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L24" s="1"/>
+      <c r="M24" s="1"/>
+      <c r="N24" s="1"/>
+      <c r="O24" s="44"/>
+      <c r="P24" s="1"/>
+      <c r="Q24" s="1"/>
+      <c r="R24" s="1"/>
+      <c r="S24" s="1"/>
+      <c r="T24" s="1"/>
+      <c r="U24" s="1"/>
+      <c r="V24" s="1"/>
+      <c r="W24" s="1"/>
+      <c r="X24" s="1"/>
+    </row>
+    <row r="25" spans="1:24" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1"/>
-      <c r="B25" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C25" s="6">
-        <v>250000</v>
-      </c>
-      <c r="D25" s="1"/>
-      <c r="E25" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="F25" s="1"/>
-      <c r="G25" s="1"/>
-      <c r="H25" s="1"/>
-      <c r="I25" s="1"/>
-      <c r="J25" s="1"/>
-      <c r="K25" s="1"/>
-    </row>
-    <row r="26" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B25" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="C25" s="8"/>
+      <c r="D25" s="8"/>
+      <c r="E25" s="38">
+        <f>E24</f>
+        <v>50000000</v>
+      </c>
+      <c r="F25" s="8"/>
+      <c r="G25" s="8"/>
+      <c r="H25" s="8"/>
+      <c r="I25" s="8"/>
+      <c r="J25" s="38">
+        <f>J24+I21</f>
+        <v>80000000</v>
+      </c>
+      <c r="K25" s="8"/>
+      <c r="L25" s="8"/>
+      <c r="M25" s="8"/>
+      <c r="N25" s="8"/>
+      <c r="O25" s="45"/>
+      <c r="P25" s="1"/>
+      <c r="Q25" s="1"/>
+      <c r="R25" s="1"/>
+      <c r="S25" s="1"/>
+      <c r="T25" s="1"/>
+      <c r="U25" s="1"/>
+      <c r="V25" s="1"/>
+      <c r="W25" s="1"/>
+      <c r="X25" s="1"/>
+    </row>
+    <row r="26" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
-      <c r="C26" s="8"/>
+      <c r="C26" s="1"/>
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
@@ -2234,16 +3572,26 @@
       <c r="I26" s="1"/>
       <c r="J26" s="1"/>
       <c r="K26" s="1"/>
-    </row>
-    <row r="27" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="L26" s="1"/>
+      <c r="M26" s="1"/>
+      <c r="N26" s="1"/>
+      <c r="O26" s="1"/>
+      <c r="P26" s="1"/>
+      <c r="Q26" s="1"/>
+      <c r="R26" s="1"/>
+      <c r="S26" s="1"/>
+      <c r="T26" s="1"/>
+      <c r="U26" s="1"/>
+      <c r="V26" s="1"/>
+      <c r="W26" s="1"/>
+      <c r="X26" s="1"/>
+    </row>
+    <row r="27" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A27" s="1"/>
-      <c r="B27" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="C27" s="5">
-        <f>SUM(C4:C25)</f>
-        <v>9825000</v>
-      </c>
+      <c r="B27" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="C27" s="1"/>
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
@@ -2252,6 +3600,195 @@
       <c r="I27" s="1"/>
       <c r="J27" s="1"/>
       <c r="K27" s="1"/>
+      <c r="L27" s="1"/>
+      <c r="M27" s="1"/>
+      <c r="N27" s="1"/>
+      <c r="O27" s="1"/>
+      <c r="P27" s="1"/>
+      <c r="Q27" s="1"/>
+      <c r="R27" s="1"/>
+      <c r="S27" s="1"/>
+      <c r="T27" s="1"/>
+      <c r="U27" s="1"/>
+      <c r="V27" s="1"/>
+      <c r="W27" s="1"/>
+      <c r="X27" s="1"/>
+    </row>
+    <row r="28" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A28" s="1"/>
+      <c r="B28" s="1"/>
+      <c r="C28" s="1"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1"/>
+      <c r="F28" s="1"/>
+      <c r="G28" s="1"/>
+      <c r="H28" s="1"/>
+      <c r="I28" s="1"/>
+      <c r="J28" s="1"/>
+      <c r="K28" s="1"/>
+      <c r="L28" s="1"/>
+      <c r="M28" s="1"/>
+      <c r="N28" s="1"/>
+      <c r="O28" s="1"/>
+      <c r="P28" s="1"/>
+      <c r="Q28" s="1"/>
+      <c r="R28" s="1"/>
+      <c r="S28" s="1"/>
+      <c r="T28" s="1"/>
+      <c r="U28" s="1"/>
+      <c r="V28" s="1"/>
+      <c r="W28" s="1"/>
+      <c r="X28" s="1"/>
+    </row>
+    <row r="29" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A29" s="1"/>
+      <c r="B29" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C29" s="2">
+        <f>J24/E24-1</f>
+        <v>0.19999999999999996</v>
+      </c>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1"/>
+      <c r="F29" s="1"/>
+      <c r="G29" s="1"/>
+      <c r="H29" s="1"/>
+      <c r="I29" s="1"/>
+      <c r="J29" s="1"/>
+      <c r="K29" s="1"/>
+      <c r="L29" s="1"/>
+      <c r="M29" s="1"/>
+      <c r="N29" s="1"/>
+      <c r="O29" s="1"/>
+      <c r="P29" s="1"/>
+      <c r="Q29" s="1"/>
+      <c r="R29" s="1"/>
+      <c r="S29" s="1"/>
+      <c r="T29" s="1"/>
+      <c r="U29" s="1"/>
+      <c r="V29" s="1"/>
+      <c r="W29" s="1"/>
+      <c r="X29" s="1"/>
+    </row>
+    <row r="30" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A30" s="1"/>
+      <c r="B30" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C30" s="37">
+        <f>'SAFE Investments'!C27</f>
+        <v>9825000</v>
+      </c>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+      <c r="F30" s="1"/>
+      <c r="G30" s="1"/>
+      <c r="H30" s="1"/>
+      <c r="I30" s="1"/>
+      <c r="J30" s="1"/>
+      <c r="K30" s="1"/>
+      <c r="L30" s="1"/>
+      <c r="M30" s="1"/>
+      <c r="N30" s="1"/>
+      <c r="O30" s="1"/>
+      <c r="P30" s="1"/>
+      <c r="Q30" s="1"/>
+      <c r="R30" s="1"/>
+      <c r="S30" s="1"/>
+      <c r="T30" s="1"/>
+      <c r="U30" s="1"/>
+      <c r="V30" s="1"/>
+      <c r="W30" s="1"/>
+      <c r="X30" s="1"/>
+    </row>
+    <row r="31" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A31" s="1"/>
+      <c r="B31" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C31" s="2">
+        <f>I21/J25</f>
+        <v>0.25</v>
+      </c>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1"/>
+      <c r="F31" s="1"/>
+      <c r="G31" s="1"/>
+      <c r="H31" s="1"/>
+      <c r="I31" s="1"/>
+      <c r="J31" s="1"/>
+      <c r="K31" s="1"/>
+      <c r="L31" s="1"/>
+      <c r="M31" s="1"/>
+      <c r="N31" s="1"/>
+      <c r="O31" s="1"/>
+      <c r="P31" s="1"/>
+      <c r="Q31" s="1"/>
+      <c r="R31" s="1"/>
+      <c r="S31" s="1"/>
+      <c r="T31" s="1"/>
+      <c r="U31" s="1"/>
+      <c r="V31" s="1"/>
+      <c r="W31" s="1"/>
+      <c r="X31" s="1"/>
+    </row>
+    <row r="32" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A32" s="1"/>
+      <c r="B32" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C32" s="3">
+        <f>0.1</f>
+        <v>0.1</v>
+      </c>
+      <c r="D32" s="1"/>
+      <c r="E32" s="1"/>
+      <c r="F32" s="1"/>
+      <c r="G32" s="1"/>
+      <c r="H32" s="1"/>
+      <c r="I32" s="1"/>
+      <c r="J32" s="1"/>
+      <c r="K32" s="1"/>
+      <c r="L32" s="1"/>
+      <c r="M32" s="1"/>
+      <c r="N32" s="1"/>
+      <c r="O32" s="1"/>
+      <c r="P32" s="1"/>
+      <c r="Q32" s="1"/>
+      <c r="R32" s="1"/>
+      <c r="S32" s="1"/>
+      <c r="T32" s="1"/>
+      <c r="U32" s="1"/>
+      <c r="V32" s="1"/>
+      <c r="W32" s="1"/>
+      <c r="X32" s="1"/>
+    </row>
+    <row r="33" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A33" s="1"/>
+      <c r="B33" s="1"/>
+      <c r="C33" s="1"/>
+      <c r="D33" s="1"/>
+      <c r="E33" s="1"/>
+      <c r="F33" s="1"/>
+      <c r="G33" s="1"/>
+      <c r="H33" s="1"/>
+      <c r="I33" s="1"/>
+      <c r="J33" s="1"/>
+      <c r="K33" s="1"/>
+      <c r="L33" s="1"/>
+      <c r="M33" s="1"/>
+      <c r="N33" s="1"/>
+      <c r="O33" s="1"/>
+      <c r="P33" s="1"/>
+      <c r="Q33" s="1"/>
+      <c r="R33" s="1"/>
+      <c r="S33" s="1"/>
+      <c r="T33" s="1"/>
+      <c r="U33" s="1"/>
+      <c r="V33" s="1"/>
+      <c r="W33" s="1"/>
+      <c r="X33" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Checkpoint: Series A cap table
</commit_message>
<xml_diff>
--- a/runs/20260415-101320/models/model.xlsx
+++ b/runs/20260415-101320/models/model.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/var/folders/pk/d3fxz1r57v334zbrzvw1g9pw0000gn/T/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E314BFD2-3A77-024B-A638-F10A7771FE1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{840AD00B-917C-094D-ABB2-DD2DFE90ACFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet8" sheetId="158" r:id="rId1"/>
     <sheet name="DetailedCapTable" sheetId="159" r:id="rId2"/>
     <sheet name="SAFE Investments" sheetId="160" r:id="rId3"/>
+    <sheet name="Series A" sheetId="161" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029" iterate="1"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="87">
   <si>
     <t>Total</t>
   </si>
@@ -193,17 +194,122 @@
     <t>Mark Lotke</t>
   </si>
   <si>
+    <t xml:space="preserve">Common </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Option </t>
+  </si>
+  <si>
+    <t>Series A</t>
+  </si>
+  <si>
+    <t>Total Capitalization</t>
+  </si>
+  <si>
+    <t># of</t>
+  </si>
+  <si>
+    <t>$</t>
+  </si>
+  <si>
+    <t>Preferred</t>
+  </si>
+  <si>
+    <t>Pool +</t>
+  </si>
+  <si>
+    <t>Total FD</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t>Shares</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Invested</t>
+  </si>
+  <si>
+    <t>FD</t>
+  </si>
+  <si>
+    <t>Common Stock and Options:</t>
+  </si>
+  <si>
+    <t>Total Common</t>
+  </si>
+  <si>
+    <t>Preferred Rounds</t>
+  </si>
+  <si>
+    <t>Totals</t>
+  </si>
+  <si>
+    <t>Price per Share</t>
+  </si>
+  <si>
+    <t>Pre-Money Valuation</t>
+  </si>
+  <si>
+    <t>Post-Money Valuation</t>
+  </si>
+  <si>
+    <t>Series A Assumptions:</t>
+  </si>
+  <si>
+    <t>SAFE Post-Money Valuation Cap</t>
+  </si>
+  <si>
+    <t>Pre SAFE</t>
+  </si>
+  <si>
+    <t>ESOP Available</t>
+  </si>
+  <si>
+    <t>Other Series A</t>
+  </si>
+  <si>
+    <t>Option Pool Expansion</t>
+  </si>
+  <si>
+    <t>Other Common Holders</t>
+  </si>
+  <si>
     <t>Transfer from Owl Rocl Capital II, LLC (Accomplice)</t>
+  </si>
+  <si>
+    <t>Small SAFE Investors</t>
+  </si>
+  <si>
+    <t>Option Pool Target %</t>
+  </si>
+  <si>
+    <t>SIDEKICK &amp; TEN ELEVEN SERIES A</t>
+  </si>
+  <si>
+    <t>SIDEKICK &amp; TEN ELEVEN</t>
+  </si>
+  <si>
+    <t>1011 (Ten Eleven)</t>
+  </si>
+  <si>
+    <t>Series A Pre-Money Valuation</t>
+  </si>
+  <si>
+    <t>Series A New Money</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="171" formatCode="&quot;$&quot;#,##0_);\(&quot;$&quot;#,##0\);&quot;$&quot;#,##0_);@_)"/>
+    <numFmt numFmtId="175" formatCode="_-[$$-409]* #,##0.0000_-;_-[$$-409]* \(#,##0.0000\)_-;_-[$$-409]* &quot;-&quot;??;_-@_-"/>
   </numFmts>
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -339,6 +445,31 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF008000"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
+    <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
@@ -364,8 +495,15 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Garamond"/>
+      <family val="1"/>
+    </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -545,8 +683,14 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -661,6 +805,147 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -706,41 +991,106 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="18" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="18" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="171" fontId="18" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="171" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="171" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="165" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="21" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="3" fontId="26" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="26" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="171" fontId="26" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="26" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="171" fontId="21" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="175" fontId="21" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1160,610 +1510,610 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
+      <c r="A1" s="8"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
+      <c r="L1" s="8"/>
+      <c r="M1" s="8"/>
+      <c r="N1" s="8"/>
+      <c r="O1" s="8"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="5" t="s">
+      <c r="A2" s="8"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="I2" s="2"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-      <c r="L2" s="1"/>
-      <c r="M2" s="1"/>
-      <c r="N2" s="1"/>
-      <c r="O2" s="1"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+      <c r="L2" s="8"/>
+      <c r="M2" s="8"/>
+      <c r="N2" s="8"/>
+      <c r="O2" s="8"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A3" s="1"/>
-      <c r="B3" s="5" t="s">
+      <c r="A3" s="8"/>
+      <c r="B3" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="18" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="18" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="5" t="s">
+      <c r="F3" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="H3" s="5" t="s">
+      <c r="H3" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="2"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
-      <c r="L3" s="1"/>
-      <c r="M3" s="1"/>
-      <c r="N3" s="1"/>
-      <c r="O3" s="1"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="8"/>
+      <c r="L3" s="8"/>
+      <c r="M3" s="8"/>
+      <c r="N3" s="8"/>
+      <c r="O3" s="8"/>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A4" s="1"/>
-      <c r="B4" s="4" t="s">
+      <c r="A4" s="8"/>
+      <c r="B4" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="19">
         <v>3600000</v>
       </c>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9"/>
-      <c r="G4" s="6">
+      <c r="D4" s="36"/>
+      <c r="E4" s="36"/>
+      <c r="F4" s="36"/>
+      <c r="G4" s="19">
         <f>SUM(C4:F4)</f>
         <v>3600000</v>
       </c>
-      <c r="H4" s="7">
+      <c r="H4" s="20">
         <f>G4/$G$23</f>
         <v>0.36959987630724139</v>
       </c>
-      <c r="I4" s="3"/>
-      <c r="J4" s="1"/>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1"/>
-      <c r="M4" s="1"/>
-      <c r="N4" s="1"/>
-      <c r="O4" s="1"/>
+      <c r="I4" s="10"/>
+      <c r="J4" s="8"/>
+      <c r="K4" s="8"/>
+      <c r="L4" s="8"/>
+      <c r="M4" s="8"/>
+      <c r="N4" s="8"/>
+      <c r="O4" s="8"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A5" s="1"/>
-      <c r="B5" s="4" t="s">
+      <c r="A5" s="8"/>
+      <c r="B5" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="6">
+      <c r="C5" s="19">
         <v>3600000</v>
       </c>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="6">
+      <c r="D5" s="36"/>
+      <c r="E5" s="36"/>
+      <c r="F5" s="36"/>
+      <c r="G5" s="19">
         <f>SUM(C5:F5)</f>
         <v>3600000</v>
       </c>
-      <c r="H5" s="7">
+      <c r="H5" s="20">
         <f>G5/$G$23</f>
         <v>0.36959987630724139</v>
       </c>
-      <c r="I5" s="3"/>
-      <c r="J5" s="1"/>
-      <c r="K5" s="1"/>
-      <c r="L5" s="1"/>
-      <c r="M5" s="1"/>
-      <c r="N5" s="1"/>
-      <c r="O5" s="1"/>
+      <c r="I5" s="10"/>
+      <c r="J5" s="8"/>
+      <c r="K5" s="8"/>
+      <c r="L5" s="8"/>
+      <c r="M5" s="8"/>
+      <c r="N5" s="8"/>
+      <c r="O5" s="8"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A6" s="1"/>
-      <c r="B6" s="4" t="s">
+      <c r="A6" s="8"/>
+      <c r="B6" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="19">
         <v>222187</v>
       </c>
-      <c r="D6" s="9"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="9"/>
-      <c r="G6" s="6">
+      <c r="D6" s="36"/>
+      <c r="E6" s="36"/>
+      <c r="F6" s="36"/>
+      <c r="G6" s="19">
         <f>SUM(C6:F6)</f>
         <v>222187</v>
       </c>
-      <c r="H6" s="7">
+      <c r="H6" s="20">
         <f>G6/$G$23</f>
         <v>2.28111910325214E-2</v>
       </c>
-      <c r="I6" s="3"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
-      <c r="L6" s="1"/>
-      <c r="M6" s="1"/>
-      <c r="N6" s="1"/>
-      <c r="O6" s="1"/>
+      <c r="I6" s="10"/>
+      <c r="J6" s="8"/>
+      <c r="K6" s="8"/>
+      <c r="L6" s="8"/>
+      <c r="M6" s="8"/>
+      <c r="N6" s="8"/>
+      <c r="O6" s="8"/>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A7" s="1"/>
-      <c r="B7" s="4" t="s">
+      <c r="A7" s="8"/>
+      <c r="B7" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="6">
+      <c r="C7" s="19">
         <v>592500</v>
       </c>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="6">
+      <c r="D7" s="36"/>
+      <c r="E7" s="36"/>
+      <c r="F7" s="36"/>
+      <c r="G7" s="19">
         <f>SUM(C7:F7)</f>
         <v>592500</v>
       </c>
-      <c r="H7" s="7">
+      <c r="H7" s="20">
         <f>G7/$G$23</f>
         <v>6.0829979642233481E-2</v>
       </c>
-      <c r="I7" s="3"/>
-      <c r="J7" s="1"/>
-      <c r="K7" s="1"/>
-      <c r="L7" s="1"/>
-      <c r="M7" s="1"/>
-      <c r="N7" s="1"/>
-      <c r="O7" s="1"/>
+      <c r="I7" s="10"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="8"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A8" s="1"/>
-      <c r="B8" s="4" t="s">
+      <c r="A8" s="8"/>
+      <c r="B8" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="6">
+      <c r="C8" s="19">
         <v>592500</v>
       </c>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="6">
+      <c r="D8" s="36"/>
+      <c r="E8" s="36"/>
+      <c r="F8" s="36"/>
+      <c r="G8" s="19">
         <f>SUM(C8:F8)</f>
         <v>592500</v>
       </c>
-      <c r="H8" s="7">
+      <c r="H8" s="20">
         <f>G8/$G$23</f>
         <v>6.0829979642233481E-2</v>
       </c>
-      <c r="I8" s="3"/>
-      <c r="J8" s="1"/>
-      <c r="K8" s="1"/>
-      <c r="L8" s="1"/>
-      <c r="M8" s="1"/>
-      <c r="N8" s="1"/>
-      <c r="O8" s="1"/>
+      <c r="I8" s="10"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A9" s="1"/>
-      <c r="B9" s="4" t="s">
+      <c r="A9" s="8"/>
+      <c r="B9" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="6">
+      <c r="C9" s="19">
         <v>13500</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="19">
         <v>98900</v>
       </c>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="6">
+      <c r="E9" s="36"/>
+      <c r="F9" s="36"/>
+      <c r="G9" s="19">
         <f>SUM(C9:F9)</f>
         <v>112400</v>
       </c>
-      <c r="H9" s="7">
+      <c r="H9" s="20">
         <f>G9/$G$23</f>
         <v>1.1539729471370537E-2</v>
       </c>
-      <c r="I9" s="3"/>
-      <c r="J9" s="1"/>
-      <c r="K9" s="1"/>
-      <c r="L9" s="1"/>
-      <c r="M9" s="1"/>
-      <c r="N9" s="1"/>
-      <c r="O9" s="1"/>
+      <c r="I9" s="10"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="8"/>
+      <c r="N9" s="8"/>
+      <c r="O9" s="8"/>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A10" s="1"/>
-      <c r="B10" s="4" t="s">
+      <c r="A10" s="8"/>
+      <c r="B10" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="6">
+      <c r="C10" s="19">
         <v>9000</v>
       </c>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="9"/>
-      <c r="G10" s="6">
+      <c r="D10" s="36"/>
+      <c r="E10" s="36"/>
+      <c r="F10" s="36"/>
+      <c r="G10" s="19">
         <f>SUM(C10:F10)</f>
         <v>9000</v>
       </c>
-      <c r="H10" s="7">
+      <c r="H10" s="20">
         <f>G10/$G$23</f>
         <v>9.2399969076810353E-4</v>
       </c>
-      <c r="I10" s="3"/>
-      <c r="J10" s="1"/>
-      <c r="K10" s="1"/>
-      <c r="L10" s="1"/>
-      <c r="M10" s="1"/>
-      <c r="N10" s="1"/>
-      <c r="O10" s="1"/>
+      <c r="I10" s="10"/>
+      <c r="J10" s="8"/>
+      <c r="K10" s="8"/>
+      <c r="L10" s="8"/>
+      <c r="M10" s="8"/>
+      <c r="N10" s="8"/>
+      <c r="O10" s="8"/>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A11" s="1"/>
-      <c r="B11" s="4" t="s">
+      <c r="A11" s="8"/>
+      <c r="B11" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="9"/>
-      <c r="D11" s="6">
+      <c r="C11" s="36"/>
+      <c r="D11" s="19">
         <v>95000</v>
       </c>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="6">
+      <c r="E11" s="36"/>
+      <c r="F11" s="36"/>
+      <c r="G11" s="19">
         <f>SUM(C11:F11)</f>
         <v>95000</v>
       </c>
-      <c r="H11" s="7">
+      <c r="H11" s="20">
         <f>G11/$G$23</f>
         <v>9.7533300692188695E-3</v>
       </c>
-      <c r="I11" s="3"/>
-      <c r="J11" s="1"/>
-      <c r="K11" s="1"/>
-      <c r="L11" s="1"/>
-      <c r="M11" s="1"/>
-      <c r="N11" s="1"/>
-      <c r="O11" s="1"/>
+      <c r="I11" s="10"/>
+      <c r="J11" s="8"/>
+      <c r="K11" s="8"/>
+      <c r="L11" s="8"/>
+      <c r="M11" s="8"/>
+      <c r="N11" s="8"/>
+      <c r="O11" s="8"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A12" s="1"/>
-      <c r="B12" s="4" t="s">
+      <c r="A12" s="8"/>
+      <c r="B12" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="6">
+      <c r="C12" s="36"/>
+      <c r="D12" s="36"/>
+      <c r="E12" s="19">
         <v>25000</v>
       </c>
-      <c r="F12" s="9"/>
-      <c r="G12" s="6">
+      <c r="F12" s="36"/>
+      <c r="G12" s="19">
         <f>SUM(C12:F12)</f>
         <v>25000</v>
       </c>
-      <c r="H12" s="7">
+      <c r="H12" s="20">
         <f>G12/$G$23</f>
         <v>2.5666658076891765E-3</v>
       </c>
-      <c r="I12" s="3"/>
-      <c r="J12" s="1"/>
-      <c r="K12" s="1"/>
-      <c r="L12" s="1"/>
-      <c r="M12" s="1"/>
-      <c r="N12" s="1"/>
-      <c r="O12" s="1"/>
+      <c r="I12" s="10"/>
+      <c r="J12" s="8"/>
+      <c r="K12" s="8"/>
+      <c r="L12" s="8"/>
+      <c r="M12" s="8"/>
+      <c r="N12" s="8"/>
+      <c r="O12" s="8"/>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A13" s="1"/>
-      <c r="B13" s="4" t="s">
+      <c r="A13" s="8"/>
+      <c r="B13" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="6">
+      <c r="C13" s="36"/>
+      <c r="D13" s="36"/>
+      <c r="E13" s="19">
         <v>41562</v>
       </c>
-      <c r="F13" s="9"/>
-      <c r="G13" s="6">
+      <c r="F13" s="36"/>
+      <c r="G13" s="19">
         <f>SUM(C13:F13)</f>
         <v>41562</v>
       </c>
-      <c r="H13" s="7">
+      <c r="H13" s="20">
         <f>G13/$G$23</f>
         <v>4.2670305719671019E-3</v>
       </c>
-      <c r="I13" s="3"/>
-      <c r="J13" s="1"/>
-      <c r="K13" s="1"/>
-      <c r="L13" s="1"/>
-      <c r="M13" s="1"/>
-      <c r="N13" s="1"/>
-      <c r="O13" s="1"/>
+      <c r="I13" s="10"/>
+      <c r="J13" s="8"/>
+      <c r="K13" s="8"/>
+      <c r="L13" s="8"/>
+      <c r="M13" s="8"/>
+      <c r="N13" s="8"/>
+      <c r="O13" s="8"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A14" s="1"/>
-      <c r="B14" s="4" t="s">
+      <c r="A14" s="8"/>
+      <c r="B14" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="C14" s="9"/>
-      <c r="D14" s="6">
+      <c r="C14" s="36"/>
+      <c r="D14" s="19">
         <v>285000</v>
       </c>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="6">
+      <c r="E14" s="36"/>
+      <c r="F14" s="36"/>
+      <c r="G14" s="19">
         <f>SUM(C14:F14)</f>
         <v>285000</v>
       </c>
-      <c r="H14" s="7">
+      <c r="H14" s="20">
         <f>G14/$G$23</f>
         <v>2.925999020765661E-2</v>
       </c>
-      <c r="I14" s="3"/>
-      <c r="J14" s="1"/>
-      <c r="K14" s="1"/>
-      <c r="L14" s="1"/>
-      <c r="M14" s="1"/>
-      <c r="N14" s="1"/>
-      <c r="O14" s="1"/>
+      <c r="I14" s="10"/>
+      <c r="J14" s="8"/>
+      <c r="K14" s="8"/>
+      <c r="L14" s="8"/>
+      <c r="M14" s="8"/>
+      <c r="N14" s="8"/>
+      <c r="O14" s="8"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A15" s="1"/>
-      <c r="B15" s="4" t="s">
+      <c r="A15" s="8"/>
+      <c r="B15" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="C15" s="9"/>
-      <c r="D15" s="6">
+      <c r="C15" s="36"/>
+      <c r="D15" s="19">
         <v>50000</v>
       </c>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9"/>
-      <c r="G15" s="6">
+      <c r="E15" s="36"/>
+      <c r="F15" s="36"/>
+      <c r="G15" s="19">
         <f>SUM(C15:F15)</f>
         <v>50000</v>
       </c>
-      <c r="H15" s="7">
+      <c r="H15" s="20">
         <f>G15/$G$23</f>
         <v>5.133331615378353E-3</v>
       </c>
-      <c r="I15" s="3"/>
-      <c r="J15" s="1"/>
-      <c r="K15" s="1"/>
-      <c r="L15" s="1"/>
-      <c r="M15" s="1"/>
-      <c r="N15" s="1"/>
-      <c r="O15" s="1"/>
+      <c r="I15" s="10"/>
+      <c r="J15" s="8"/>
+      <c r="K15" s="8"/>
+      <c r="L15" s="8"/>
+      <c r="M15" s="8"/>
+      <c r="N15" s="8"/>
+      <c r="O15" s="8"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A16" s="1"/>
-      <c r="B16" s="4" t="s">
+      <c r="A16" s="8"/>
+      <c r="B16" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="C16" s="9"/>
-      <c r="D16" s="6">
+      <c r="C16" s="36"/>
+      <c r="D16" s="19">
         <v>285000</v>
       </c>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="6">
+      <c r="E16" s="36"/>
+      <c r="F16" s="36"/>
+      <c r="G16" s="19">
         <f>SUM(C16:F16)</f>
         <v>285000</v>
       </c>
-      <c r="H16" s="7">
+      <c r="H16" s="20">
         <f>G16/$G$23</f>
         <v>2.925999020765661E-2</v>
       </c>
-      <c r="I16" s="3"/>
-      <c r="J16" s="1"/>
-      <c r="K16" s="1"/>
-      <c r="L16" s="1"/>
-      <c r="M16" s="1"/>
-      <c r="N16" s="1"/>
-      <c r="O16" s="1"/>
+      <c r="I16" s="10"/>
+      <c r="J16" s="8"/>
+      <c r="K16" s="8"/>
+      <c r="L16" s="8"/>
+      <c r="M16" s="8"/>
+      <c r="N16" s="8"/>
+      <c r="O16" s="8"/>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A17" s="1"/>
-      <c r="B17" s="4" t="s">
+      <c r="A17" s="8"/>
+      <c r="B17" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="9"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="6">
+      <c r="C17" s="36"/>
+      <c r="D17" s="36"/>
+      <c r="E17" s="19">
         <v>96186</v>
       </c>
-      <c r="F17" s="9"/>
-      <c r="G17" s="6">
+      <c r="F17" s="36"/>
+      <c r="G17" s="19">
         <f>SUM(C17:F17)</f>
         <v>96186</v>
       </c>
-      <c r="H17" s="7">
+      <c r="H17" s="20">
         <f>G17/$G$23</f>
         <v>9.8750926951356455E-3</v>
       </c>
-      <c r="I17" s="3"/>
-      <c r="J17" s="1"/>
-      <c r="K17" s="1"/>
-      <c r="L17" s="1"/>
-      <c r="M17" s="1"/>
-      <c r="N17" s="1"/>
-      <c r="O17" s="1"/>
+      <c r="I17" s="10"/>
+      <c r="J17" s="8"/>
+      <c r="K17" s="8"/>
+      <c r="L17" s="8"/>
+      <c r="M17" s="8"/>
+      <c r="N17" s="8"/>
+      <c r="O17" s="8"/>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A18" s="1"/>
-      <c r="B18" s="4" t="s">
+      <c r="A18" s="8"/>
+      <c r="B18" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="C18" s="9"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="6">
+      <c r="C18" s="36"/>
+      <c r="D18" s="36"/>
+      <c r="E18" s="19">
         <v>48095</v>
       </c>
-      <c r="F18" s="9"/>
-      <c r="G18" s="6">
+      <c r="F18" s="36"/>
+      <c r="G18" s="19">
         <f>SUM(C18:F18)</f>
         <v>48095</v>
       </c>
-      <c r="H18" s="7">
+      <c r="H18" s="20">
         <f>G18/$G$23</f>
         <v>4.9377516808324371E-3</v>
       </c>
-      <c r="I18" s="3"/>
-      <c r="J18" s="1"/>
-      <c r="K18" s="1"/>
-      <c r="L18" s="1"/>
-      <c r="M18" s="1"/>
-      <c r="N18" s="1"/>
-      <c r="O18" s="1"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="8"/>
+      <c r="K18" s="8"/>
+      <c r="L18" s="8"/>
+      <c r="M18" s="8"/>
+      <c r="N18" s="8"/>
+      <c r="O18" s="8"/>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A19" s="1"/>
-      <c r="B19" s="4" t="s">
+      <c r="A19" s="8"/>
+      <c r="B19" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="6">
+      <c r="C19" s="36"/>
+      <c r="D19" s="36"/>
+      <c r="E19" s="36"/>
+      <c r="F19" s="19">
         <v>12395</v>
       </c>
-      <c r="G19" s="6">
+      <c r="G19" s="19">
         <f>SUM(C19:F19)</f>
         <v>12395</v>
       </c>
-      <c r="H19" s="7">
+      <c r="H19" s="20">
         <f>G19/$G$23</f>
         <v>1.2725529074522936E-3</v>
       </c>
-      <c r="I19" s="3"/>
-      <c r="J19" s="1"/>
-      <c r="K19" s="1"/>
-      <c r="L19" s="1"/>
-      <c r="M19" s="1"/>
-      <c r="N19" s="1"/>
-      <c r="O19" s="1"/>
+      <c r="I19" s="10"/>
+      <c r="J19" s="8"/>
+      <c r="K19" s="8"/>
+      <c r="L19" s="8"/>
+      <c r="M19" s="8"/>
+      <c r="N19" s="8"/>
+      <c r="O19" s="8"/>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A20" s="1"/>
-      <c r="B20" s="4" t="s">
+      <c r="A20" s="8"/>
+      <c r="B20" s="17" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="9"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="6">
+      <c r="C20" s="36"/>
+      <c r="D20" s="36"/>
+      <c r="E20" s="36"/>
+      <c r="F20" s="19">
         <v>8333</v>
       </c>
-      <c r="G20" s="6">
+      <c r="G20" s="19">
         <f>SUM(C20:F20)</f>
         <v>8333</v>
       </c>
-      <c r="H20" s="7">
+      <c r="H20" s="20">
         <f>G20/$G$23</f>
         <v>8.5552104701895626E-4</v>
       </c>
-      <c r="I20" s="3"/>
-      <c r="J20" s="1"/>
-      <c r="K20" s="1"/>
-      <c r="L20" s="1"/>
-      <c r="M20" s="1"/>
-      <c r="N20" s="1"/>
-      <c r="O20" s="1"/>
+      <c r="I20" s="10"/>
+      <c r="J20" s="8"/>
+      <c r="K20" s="8"/>
+      <c r="L20" s="8"/>
+      <c r="M20" s="8"/>
+      <c r="N20" s="8"/>
+      <c r="O20" s="8"/>
     </row>
     <row r="21" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="1"/>
-      <c r="B21" s="4" t="s">
+      <c r="A21" s="8"/>
+      <c r="B21" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="C21" s="9"/>
-      <c r="D21" s="6">
+      <c r="C21" s="36"/>
+      <c r="D21" s="19">
         <v>65105</v>
       </c>
-      <c r="E21" s="9"/>
-      <c r="F21" s="9"/>
-      <c r="G21" s="6">
+      <c r="E21" s="36"/>
+      <c r="F21" s="36"/>
+      <c r="G21" s="19">
         <f>SUM(C21:F21)</f>
         <v>65105</v>
       </c>
-      <c r="H21" s="7">
+      <c r="H21" s="20">
         <f>G21/$G$23</f>
         <v>6.6841110963841528E-3</v>
       </c>
-      <c r="I21" s="3"/>
-      <c r="J21" s="1"/>
-      <c r="K21" s="1"/>
-      <c r="L21" s="1"/>
-      <c r="M21" s="1"/>
-      <c r="N21" s="1"/>
-      <c r="O21" s="1"/>
+      <c r="I21" s="10"/>
+      <c r="J21" s="8"/>
+      <c r="K21" s="8"/>
+      <c r="L21" s="8"/>
+      <c r="M21" s="8"/>
+      <c r="N21" s="8"/>
+      <c r="O21" s="8"/>
     </row>
     <row r="22" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="9"/>
-      <c r="H22" s="3"/>
-      <c r="I22" s="3"/>
-      <c r="J22" s="1"/>
-      <c r="K22" s="1"/>
-      <c r="L22" s="1"/>
-      <c r="M22" s="1"/>
-      <c r="N22" s="1"/>
-      <c r="O22" s="1"/>
+      <c r="A22" s="8"/>
+      <c r="B22" s="8"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
+      <c r="G22" s="36"/>
+      <c r="H22" s="10"/>
+      <c r="I22" s="10"/>
+      <c r="J22" s="8"/>
+      <c r="K22" s="8"/>
+      <c r="L22" s="8"/>
+      <c r="M22" s="8"/>
+      <c r="N22" s="8"/>
+      <c r="O22" s="8"/>
     </row>
     <row r="23" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="1"/>
-      <c r="B23" s="5" t="s">
+      <c r="A23" s="8"/>
+      <c r="B23" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="C23" s="6">
+      <c r="C23" s="19">
         <f>SUM(C4:C21)</f>
         <v>8629687</v>
       </c>
-      <c r="D23" s="6">
+      <c r="D23" s="19">
         <f>SUM(D4:D21)</f>
         <v>879005</v>
       </c>
-      <c r="E23" s="6">
+      <c r="E23" s="19">
         <f>SUM(E4:E21)</f>
         <v>210843</v>
       </c>
-      <c r="F23" s="6">
+      <c r="F23" s="19">
         <f>SUM(F4:F21)</f>
         <v>20728</v>
       </c>
-      <c r="G23" s="6">
+      <c r="G23" s="19">
         <f>SUM(G4:G21)</f>
         <v>9740263</v>
       </c>
-      <c r="H23" s="9"/>
-      <c r="I23" s="9"/>
-      <c r="J23" s="1"/>
-      <c r="K23" s="1"/>
-      <c r="L23" s="1"/>
-      <c r="M23" s="1"/>
-      <c r="N23" s="1"/>
-      <c r="O23" s="1"/>
+      <c r="H23" s="36"/>
+      <c r="I23" s="36"/>
+      <c r="J23" s="8"/>
+      <c r="K23" s="8"/>
+      <c r="L23" s="8"/>
+      <c r="M23" s="8"/>
+      <c r="N23" s="8"/>
+      <c r="O23" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1785,463 +2135,1008 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A1" s="1"/>
-      <c r="B1" s="1"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
+      <c r="A1" s="8"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
+      <c r="K1" s="8"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
+      <c r="A2" s="8"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="38"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="8"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A3" s="1"/>
-      <c r="B3" s="5" t="s">
+      <c r="A3" s="8"/>
+      <c r="B3" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="D3" s="1"/>
-      <c r="E3" s="5" t="s">
+      <c r="D3" s="8"/>
+      <c r="E3" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8"/>
+      <c r="I3" s="8"/>
+      <c r="J3" s="8"/>
+      <c r="K3" s="8"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A4" s="1"/>
-      <c r="B4" s="4" t="s">
+      <c r="A4" s="8"/>
+      <c r="B4" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="8">
+      <c r="C4" s="21">
         <v>25000</v>
       </c>
-      <c r="D4" s="1"/>
-      <c r="E4" s="4" t="s">
+      <c r="D4" s="8"/>
+      <c r="E4" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="F4" s="1"/>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
-      <c r="K4" s="1"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="8"/>
+      <c r="I4" s="8"/>
+      <c r="J4" s="8"/>
+      <c r="K4" s="8"/>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
-      <c r="A5" s="1"/>
-      <c r="B5" s="4" t="s">
+      <c r="A5" s="8"/>
+      <c r="B5" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="C5" s="8">
+      <c r="C5" s="21">
         <v>25000</v>
       </c>
-      <c r="D5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
-      <c r="K5" s="1"/>
+      <c r="D5" s="8"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="8"/>
+      <c r="H5" s="8"/>
+      <c r="I5" s="8"/>
+      <c r="J5" s="8"/>
+      <c r="K5" s="8"/>
     </row>
     <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="1"/>
-      <c r="B6" s="4" t="s">
+      <c r="A6" s="8"/>
+      <c r="B6" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="8">
+      <c r="C6" s="21">
         <v>137170.75</v>
       </c>
-      <c r="D6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
+      <c r="D6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="8"/>
+      <c r="K6" s="8"/>
     </row>
     <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="1"/>
-      <c r="B7" s="4" t="s">
+      <c r="A7" s="8"/>
+      <c r="B7" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="8">
+      <c r="C7" s="21">
         <v>3846829.25</v>
       </c>
-      <c r="D7" s="1"/>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
-      <c r="K7" s="1"/>
+      <c r="D7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
     </row>
     <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="1"/>
-      <c r="B8" s="4" t="s">
+      <c r="A8" s="8"/>
+      <c r="B8" s="17" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="8">
+      <c r="C8" s="21">
         <v>16566</v>
       </c>
-      <c r="D8" s="1"/>
-      <c r="E8" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
-      <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-      <c r="J8" s="1"/>
-      <c r="K8" s="1"/>
+      <c r="D8" s="8"/>
+      <c r="E8" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
     </row>
     <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="1"/>
-      <c r="B9" s="4" t="s">
+      <c r="A9" s="8"/>
+      <c r="B9" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="8">
+      <c r="C9" s="21">
         <v>250000</v>
       </c>
-      <c r="D9" s="1"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
-      <c r="J9" s="1"/>
-      <c r="K9" s="1"/>
+      <c r="D9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
     </row>
     <row r="10" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="1"/>
-      <c r="B10" s="4" t="s">
+      <c r="A10" s="8"/>
+      <c r="B10" s="17" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="8">
+      <c r="C10" s="21">
         <v>100000</v>
       </c>
-      <c r="D10" s="1"/>
-      <c r="F10" s="1"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1"/>
-      <c r="J10" s="1"/>
-      <c r="K10" s="1"/>
+      <c r="D10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8"/>
+      <c r="K10" s="8"/>
     </row>
     <row r="11" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="1"/>
-      <c r="B11" s="4" t="s">
+      <c r="A11" s="8"/>
+      <c r="B11" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="8">
+      <c r="C11" s="21">
         <v>300000</v>
       </c>
-      <c r="D11" s="1"/>
-      <c r="E11" s="4" t="s">
+      <c r="D11" s="8"/>
+      <c r="E11" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="F11" s="1"/>
-      <c r="G11" s="1"/>
-      <c r="H11" s="1"/>
-      <c r="I11" s="1"/>
-      <c r="J11" s="1"/>
-      <c r="K11" s="1"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8"/>
+      <c r="J11" s="8"/>
+      <c r="K11" s="8"/>
     </row>
     <row r="12" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="1"/>
-      <c r="B12" s="4" t="s">
+      <c r="A12" s="8"/>
+      <c r="B12" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="C12" s="8">
+      <c r="C12" s="21">
         <v>37500</v>
       </c>
-      <c r="D12" s="1"/>
-      <c r="E12" s="4" t="s">
+      <c r="D12" s="8"/>
+      <c r="E12" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="F12" s="1"/>
-      <c r="G12" s="1"/>
-      <c r="H12" s="1"/>
-      <c r="I12" s="1"/>
-      <c r="J12" s="1"/>
-      <c r="K12" s="1"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8"/>
+      <c r="I12" s="8"/>
+      <c r="J12" s="8"/>
+      <c r="K12" s="8"/>
     </row>
     <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="1"/>
-      <c r="B13" s="4" t="s">
+      <c r="A13" s="8"/>
+      <c r="B13" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="8">
+      <c r="C13" s="21">
         <v>250000</v>
       </c>
-      <c r="D13" s="1"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
-      <c r="I13" s="1"/>
-      <c r="J13" s="1"/>
-      <c r="K13" s="1"/>
+      <c r="D13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8"/>
+      <c r="I13" s="8"/>
+      <c r="J13" s="8"/>
+      <c r="K13" s="8"/>
     </row>
     <row r="14" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="1"/>
-      <c r="B14" s="4" t="s">
+      <c r="A14" s="8"/>
+      <c r="B14" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="C14" s="8">
+      <c r="C14" s="21">
         <v>100000</v>
       </c>
-      <c r="D14" s="1"/>
-      <c r="F14" s="1"/>
-      <c r="G14" s="1"/>
-      <c r="H14" s="1"/>
-      <c r="I14" s="1"/>
-      <c r="J14" s="1"/>
-      <c r="K14" s="1"/>
+      <c r="D14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
+      <c r="J14" s="8"/>
+      <c r="K14" s="8"/>
     </row>
     <row r="15" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="1"/>
-      <c r="B15" s="4" t="s">
+      <c r="A15" s="8"/>
+      <c r="B15" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="C15" s="8">
+      <c r="C15" s="21">
         <v>41164</v>
       </c>
-      <c r="D15" s="1"/>
-      <c r="E15" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1"/>
-      <c r="J15" s="1"/>
-      <c r="K15" s="1"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="8"/>
+      <c r="J15" s="8"/>
+      <c r="K15" s="8"/>
     </row>
     <row r="16" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="1"/>
-      <c r="B16" s="4" t="s">
+      <c r="A16" s="8"/>
+      <c r="B16" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="C16" s="8">
+      <c r="C16" s="21">
         <v>2328778</v>
       </c>
-      <c r="D16" s="1"/>
-      <c r="E16" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="F16" s="1"/>
-      <c r="G16" s="1"/>
-      <c r="H16" s="1"/>
-      <c r="I16" s="1"/>
-      <c r="J16" s="1"/>
-      <c r="K16" s="1"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="8"/>
+      <c r="J16" s="8"/>
+      <c r="K16" s="8"/>
     </row>
     <row r="17" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="1"/>
-      <c r="B17" s="4" t="s">
+      <c r="A17" s="8"/>
+      <c r="B17" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="C17" s="8">
+      <c r="C17" s="21">
         <v>1506000</v>
       </c>
-      <c r="D17" s="1"/>
-      <c r="E17" s="4" t="s">
+      <c r="D17" s="8"/>
+      <c r="E17" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="F17" s="1"/>
-      <c r="G17" s="1"/>
-      <c r="H17" s="1"/>
-      <c r="I17" s="1"/>
-      <c r="J17" s="1"/>
-      <c r="K17" s="1"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="8"/>
+      <c r="K17" s="8"/>
     </row>
     <row r="18" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="1"/>
-      <c r="B18" s="4" t="s">
+      <c r="A18" s="8"/>
+      <c r="B18" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="C18" s="8">
+      <c r="C18" s="21">
         <v>50000</v>
       </c>
-      <c r="D18" s="1"/>
-      <c r="F18" s="1"/>
-      <c r="G18" s="1"/>
-      <c r="H18" s="1"/>
-      <c r="I18" s="1"/>
-      <c r="J18" s="1"/>
-      <c r="K18" s="1"/>
+      <c r="D18" s="8"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="8"/>
+      <c r="H18" s="8"/>
+      <c r="I18" s="8"/>
+      <c r="J18" s="8"/>
+      <c r="K18" s="8"/>
     </row>
     <row r="19" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="1"/>
-      <c r="B19" s="4" t="s">
+      <c r="A19" s="8"/>
+      <c r="B19" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="C19" s="8">
+      <c r="C19" s="21">
         <v>212500</v>
       </c>
-      <c r="D19" s="1"/>
-      <c r="E19" s="4" t="s">
+      <c r="D19" s="8"/>
+      <c r="E19" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="F19" s="1"/>
-      <c r="G19" s="1"/>
-      <c r="H19" s="1"/>
-      <c r="I19" s="1"/>
-      <c r="J19" s="1"/>
-      <c r="K19" s="1"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="8"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="8"/>
+      <c r="J19" s="8"/>
+      <c r="K19" s="8"/>
     </row>
     <row r="20" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="1"/>
-      <c r="B20" s="4" t="s">
+      <c r="A20" s="8"/>
+      <c r="B20" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="C20" s="8">
+      <c r="C20" s="21">
         <v>25000</v>
       </c>
-      <c r="D20" s="1"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
-      <c r="H20" s="1"/>
-      <c r="I20" s="1"/>
-      <c r="J20" s="1"/>
-      <c r="K20" s="1"/>
+      <c r="D20" s="8"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="8"/>
+      <c r="H20" s="8"/>
+      <c r="I20" s="8"/>
+      <c r="J20" s="8"/>
+      <c r="K20" s="8"/>
     </row>
     <row r="21" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="1"/>
-      <c r="B21" s="4" t="s">
+      <c r="A21" s="8"/>
+      <c r="B21" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="C21" s="8">
+      <c r="C21" s="21">
         <v>61746</v>
       </c>
-      <c r="D21" s="1"/>
-      <c r="E21" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="F21" s="1"/>
-      <c r="G21" s="1"/>
-      <c r="H21" s="1"/>
-      <c r="I21" s="1"/>
-      <c r="J21" s="1"/>
-      <c r="K21" s="1"/>
+      <c r="D21" s="8"/>
+      <c r="E21" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="F21" s="8"/>
+      <c r="G21" s="8"/>
+      <c r="H21" s="8"/>
+      <c r="I21" s="8"/>
+      <c r="J21" s="8"/>
+      <c r="K21" s="8"/>
     </row>
     <row r="22" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="1"/>
-      <c r="B22" s="4" t="s">
+      <c r="A22" s="8"/>
+      <c r="B22" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="C22" s="8">
+      <c r="C22" s="21">
         <v>100000</v>
       </c>
-      <c r="D22" s="1"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
-      <c r="H22" s="1"/>
-      <c r="I22" s="1"/>
-      <c r="J22" s="1"/>
-      <c r="K22" s="1"/>
+      <c r="D22" s="8"/>
+      <c r="F22" s="8"/>
+      <c r="G22" s="8"/>
+      <c r="H22" s="8"/>
+      <c r="I22" s="8"/>
+      <c r="J22" s="8"/>
+      <c r="K22" s="8"/>
     </row>
     <row r="23" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="1"/>
-      <c r="B23" s="4" t="s">
+      <c r="A23" s="8"/>
+      <c r="B23" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="C23" s="8">
+      <c r="C23" s="21">
         <v>100000</v>
       </c>
-      <c r="D23" s="1"/>
-      <c r="F23" s="1"/>
-      <c r="G23" s="1"/>
-      <c r="H23" s="1"/>
-      <c r="I23" s="1"/>
-      <c r="J23" s="1"/>
-      <c r="K23" s="1"/>
+      <c r="D23" s="8"/>
+      <c r="F23" s="8"/>
+      <c r="G23" s="8"/>
+      <c r="H23" s="8"/>
+      <c r="I23" s="8"/>
+      <c r="J23" s="8"/>
+      <c r="K23" s="8"/>
     </row>
     <row r="24" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="1"/>
-      <c r="B24" s="4" t="s">
+      <c r="A24" s="8"/>
+      <c r="B24" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="C24" s="8">
+      <c r="C24" s="21">
         <v>61746</v>
       </c>
-      <c r="D24" s="1"/>
-      <c r="E24" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="F24" s="1"/>
-      <c r="G24" s="1"/>
-      <c r="H24" s="1"/>
-      <c r="I24" s="1"/>
-      <c r="J24" s="1"/>
-      <c r="K24" s="1"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="F24" s="8"/>
+      <c r="G24" s="8"/>
+      <c r="H24" s="8"/>
+      <c r="I24" s="8"/>
+      <c r="J24" s="8"/>
+      <c r="K24" s="8"/>
     </row>
     <row r="25" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="1"/>
-      <c r="B25" s="4" t="s">
+      <c r="A25" s="8"/>
+      <c r="B25" s="17" t="s">
         <v>50</v>
       </c>
-      <c r="C25" s="8">
+      <c r="C25" s="21">
         <v>250000</v>
       </c>
-      <c r="D25" s="1"/>
-      <c r="E25" s="4" t="s">
+      <c r="D25" s="8"/>
+      <c r="E25" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="F25" s="1"/>
-      <c r="G25" s="1"/>
-      <c r="H25" s="1"/>
-      <c r="I25" s="1"/>
-      <c r="J25" s="1"/>
-      <c r="K25" s="1"/>
+      <c r="F25" s="8"/>
+      <c r="G25" s="8"/>
+      <c r="H25" s="8"/>
+      <c r="I25" s="8"/>
+      <c r="J25" s="8"/>
+      <c r="K25" s="8"/>
     </row>
     <row r="26" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="1"/>
-      <c r="B26" s="1"/>
-      <c r="C26" s="10"/>
-      <c r="D26" s="1"/>
-      <c r="F26" s="1"/>
-      <c r="G26" s="1"/>
-      <c r="H26" s="1"/>
-      <c r="I26" s="1"/>
-      <c r="J26" s="1"/>
-      <c r="K26" s="1"/>
+      <c r="A26" s="8"/>
+      <c r="B26" s="8"/>
+      <c r="C26" s="37"/>
+      <c r="D26" s="8"/>
+      <c r="F26" s="8"/>
+      <c r="G26" s="8"/>
+      <c r="H26" s="8"/>
+      <c r="I26" s="8"/>
+      <c r="J26" s="8"/>
+      <c r="K26" s="8"/>
     </row>
     <row r="27" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="1"/>
-      <c r="B27" s="4" t="s">
+      <c r="A27" s="8"/>
+      <c r="B27" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="C27" s="8">
+      <c r="C27" s="21">
         <f>SUM(C4:C25)</f>
         <v>9825000</v>
       </c>
-      <c r="D27" s="1"/>
-      <c r="F27" s="1"/>
-      <c r="G27" s="1"/>
-      <c r="H27" s="1"/>
-      <c r="I27" s="1"/>
-      <c r="J27" s="1"/>
-      <c r="K27" s="1"/>
+      <c r="D27" s="8"/>
+      <c r="F27" s="8"/>
+      <c r="G27" s="8"/>
+      <c r="H27" s="8"/>
+      <c r="I27" s="8"/>
+      <c r="J27" s="8"/>
+      <c r="K27" s="8"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC1D949A-8EC4-5C40-A36E-F5F8D1411C85}">
+  <dimension ref="B1:N32"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="6.33203125" customWidth="1"/>
+    <col min="2" max="2" width="35.5" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
+    <col min="4" max="4" width="17.6640625" customWidth="1"/>
+    <col min="5" max="5" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="0.5" customWidth="1"/>
+    <col min="7" max="7" width="13.83203125" customWidth="1"/>
+    <col min="8" max="8" width="0.5" customWidth="1"/>
+    <col min="9" max="9" width="17.5" customWidth="1"/>
+    <col min="10" max="10" width="16.83203125" customWidth="1"/>
+    <col min="11" max="11" width="0.5" customWidth="1"/>
+    <col min="12" max="12" width="15.5" customWidth="1"/>
+    <col min="13" max="13" width="9.33203125" customWidth="1"/>
+    <col min="14" max="14" width="6.83203125" customWidth="1"/>
+    <col min="15" max="15" width="15.5" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B1" s="11" t="s">
+        <v>83</v>
+      </c>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
+      <c r="J1" s="11"/>
+      <c r="K1" s="11"/>
+      <c r="L1" s="11"/>
+      <c r="M1" s="11"/>
+    </row>
+    <row r="2" spans="2:14" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B2" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="11"/>
+      <c r="J2" s="11"/>
+      <c r="K2" s="11"/>
+      <c r="L2" s="11"/>
+      <c r="M2" s="11"/>
+    </row>
+    <row r="3" spans="2:14" ht="16.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B3" s="5"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5"/>
+      <c r="K3" s="5"/>
+      <c r="L3" s="5"/>
+      <c r="M3" s="5"/>
+    </row>
+    <row r="4" spans="2:14" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C4" s="26" t="s">
+        <v>52</v>
+      </c>
+      <c r="D4" s="45" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" s="43"/>
+      <c r="G4" s="31" t="s">
+        <v>53</v>
+      </c>
+      <c r="I4" s="45" t="s">
+        <v>54</v>
+      </c>
+      <c r="J4" s="43"/>
+      <c r="L4" s="42" t="s">
+        <v>55</v>
+      </c>
+      <c r="M4" s="43"/>
+    </row>
+    <row r="5" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="C5" s="25" t="s">
+        <v>56</v>
+      </c>
+      <c r="D5" s="31" t="s">
+        <v>57</v>
+      </c>
+      <c r="E5" s="27" t="s">
+        <v>58</v>
+      </c>
+      <c r="G5" s="30" t="s">
+        <v>59</v>
+      </c>
+      <c r="I5" s="31" t="s">
+        <v>57</v>
+      </c>
+      <c r="J5" s="27" t="s">
+        <v>58</v>
+      </c>
+      <c r="L5" s="26" t="s">
+        <v>60</v>
+      </c>
+      <c r="M5" s="27" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="6" spans="2:14" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C6" s="28" t="s">
+        <v>62</v>
+      </c>
+      <c r="D6" s="32" t="s">
+        <v>63</v>
+      </c>
+      <c r="E6" s="29" t="s">
+        <v>62</v>
+      </c>
+      <c r="G6" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="I6" s="32" t="s">
+        <v>63</v>
+      </c>
+      <c r="J6" s="29" t="s">
+        <v>62</v>
+      </c>
+      <c r="L6" s="28" t="s">
+        <v>62</v>
+      </c>
+      <c r="M6" s="29" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="7" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B7" s="33" t="s">
+        <v>65</v>
+      </c>
+      <c r="C7" s="39"/>
+      <c r="D7" s="39"/>
+      <c r="E7" s="39"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="39"/>
+      <c r="H7" s="13"/>
+      <c r="I7" s="39"/>
+      <c r="J7" s="39"/>
+      <c r="K7" s="13"/>
+      <c r="L7" s="39"/>
+      <c r="M7" s="15"/>
+    </row>
+    <row r="8" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B8" s="34" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="2">
+        <f>DetailedCapTable!G4</f>
+        <v>3600000</v>
+      </c>
+      <c r="L8" s="22">
+        <f>C8+E8+G8+J8</f>
+        <v>3600000</v>
+      </c>
+      <c r="M8" s="41">
+        <f ca="1">L8/$L$22</f>
+        <v>0.18702070100969359</v>
+      </c>
+    </row>
+    <row r="9" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B9" s="34" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="2">
+        <f>DetailedCapTable!G5</f>
+        <v>3600000</v>
+      </c>
+      <c r="L9" s="22">
+        <f>C9+E9+G9+J9</f>
+        <v>3600000</v>
+      </c>
+      <c r="M9" s="41">
+        <f ca="1">L9/$L$22</f>
+        <v>0.18702070100969359</v>
+      </c>
+    </row>
+    <row r="10" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B10" s="34" t="s">
+        <v>78</v>
+      </c>
+      <c r="C10" s="2">
+        <f>DetailedCapTable!G23-C8-C9-G11</f>
+        <v>2475158</v>
+      </c>
+      <c r="L10" s="22">
+        <f>C10+E10+G10+J10</f>
+        <v>2475158</v>
+      </c>
+      <c r="M10" s="41">
+        <f ca="1">L10/$L$22</f>
+        <v>0.12858494007493088</v>
+      </c>
+    </row>
+    <row r="11" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B11" s="34" t="s">
+        <v>75</v>
+      </c>
+      <c r="G11" s="2">
+        <f>DetailedCapTable!G21</f>
+        <v>65105</v>
+      </c>
+      <c r="L11" s="22">
+        <f>C11+E11+G11+J11</f>
+        <v>65105</v>
+      </c>
+      <c r="M11" s="41">
+        <f ca="1">L11/$L$22</f>
+        <v>3.3822174275655839E-3</v>
+      </c>
+      <c r="N11" s="40">
+        <f ca="1">G22/L22</f>
+        <v>0.10000002078007789</v>
+      </c>
+    </row>
+    <row r="12" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B12" s="34" t="s">
+        <v>77</v>
+      </c>
+      <c r="G12" s="22">
+        <f ca="1">IFERROR(ROUND($C$32*L22-G11,0),0)</f>
+        <v>1859816</v>
+      </c>
+      <c r="L12" s="22">
+        <f ca="1">C12+E12+G12+J12</f>
+        <v>1859816</v>
+      </c>
+      <c r="M12" s="41">
+        <f ca="1">L12/$L$22</f>
+        <v>9.6617803352512313E-2</v>
+      </c>
+    </row>
+    <row r="13" spans="2:14" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B13" s="35" t="s">
+        <v>66</v>
+      </c>
+      <c r="C13" s="46">
+        <f>SUM(C8:C12)</f>
+        <v>9675158</v>
+      </c>
+      <c r="G13" s="46">
+        <f ca="1">SUM(G11:G12)</f>
+        <v>1924921</v>
+      </c>
+      <c r="L13" s="22">
+        <f ca="1">SUM(L8:L12)</f>
+        <v>11600079</v>
+      </c>
+      <c r="M13" s="41">
+        <f ca="1">L13/$L$22</f>
+        <v>0.60262636287439597</v>
+      </c>
+    </row>
+    <row r="14" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B14" s="35" t="s">
+        <v>67</v>
+      </c>
+      <c r="L14" s="22"/>
+      <c r="M14" s="41"/>
+    </row>
+    <row r="15" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B15" s="34" t="s">
+        <v>42</v>
+      </c>
+      <c r="D15" s="16">
+        <f>SUM('SAFE Investments'!C6,'SAFE Investments'!C7,'SAFE Investments'!C8,'SAFE Investments'!C15,'SAFE Investments'!C16,'SAFE Investments'!C17,'SAFE Investments'!C21,'SAFE Investments'!C24)</f>
+        <v>8000000</v>
+      </c>
+      <c r="E15" s="22">
+        <f ca="1">IFERROR(ROUND(D15/$E$24,0),0)</f>
+        <v>2309869</v>
+      </c>
+      <c r="I15" s="6">
+        <v>5000000</v>
+      </c>
+      <c r="J15" s="22">
+        <f ca="1">IFERROR(ROUND(I15/$J$24,0),0)</f>
+        <v>1203080</v>
+      </c>
+      <c r="L15" s="22">
+        <f ca="1">C15+E15+G15+J15</f>
+        <v>3512949</v>
+      </c>
+      <c r="M15" s="41">
+        <f ca="1">L15/$L$22</f>
+        <v>0.18249838460869502</v>
+      </c>
+    </row>
+    <row r="16" spans="2:14" x14ac:dyDescent="0.2">
+      <c r="B16" s="34" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16" s="16">
+        <f>'SAFE Investments'!C11</f>
+        <v>300000</v>
+      </c>
+      <c r="E16" s="22">
+        <f ca="1">IFERROR(ROUND(D16/$E$24,0),0)</f>
+        <v>86620</v>
+      </c>
+      <c r="I16" s="12"/>
+      <c r="J16" s="1"/>
+      <c r="L16" s="22">
+        <f ca="1">C16+E16+G16+J16</f>
+        <v>86620</v>
+      </c>
+      <c r="M16" s="41">
+        <f ca="1">L16/$L$22</f>
+        <v>4.4999258670721277E-3</v>
+      </c>
+    </row>
+    <row r="17" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B17" s="34" t="s">
+        <v>37</v>
+      </c>
+      <c r="D17" s="16">
+        <f>'SAFE Investments'!C13</f>
+        <v>250000</v>
+      </c>
+      <c r="E17" s="22">
+        <f ca="1">IFERROR(ROUND(D17/$E$24,0),0)</f>
+        <v>72183</v>
+      </c>
+      <c r="I17" s="12"/>
+      <c r="J17" s="1"/>
+      <c r="L17" s="22">
+        <f ca="1">C17+E17+G17+J17</f>
+        <v>72183</v>
+      </c>
+      <c r="M17" s="41">
+        <f ca="1">L17/$L$22</f>
+        <v>3.7499209058285314E-3</v>
+      </c>
+    </row>
+    <row r="18" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B18" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="D18" s="24">
+        <f>'SAFE Investments'!C27-D15-D16-D17</f>
+        <v>1275000</v>
+      </c>
+      <c r="E18" s="22">
+        <f ca="1">IFERROR(ROUND(D18/$E$24,0),0)</f>
+        <v>368135</v>
+      </c>
+      <c r="I18" s="12"/>
+      <c r="J18" s="1"/>
+      <c r="L18" s="22">
+        <f ca="1">C18+E18+G18+J18</f>
+        <v>368135</v>
+      </c>
+      <c r="M18" s="41">
+        <f ca="1">L18/$L$22</f>
+        <v>1.9124684935056542E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B19" s="34" t="s">
+        <v>84</v>
+      </c>
+      <c r="D19" s="12"/>
+      <c r="E19" s="1"/>
+      <c r="I19" s="6">
+        <v>12000000</v>
+      </c>
+      <c r="J19" s="22">
+        <f ca="1">IFERROR(ROUND(I19/$J$24,0),0)</f>
+        <v>2887392</v>
+      </c>
+      <c r="L19" s="22">
+        <f ca="1">C19+E19+G19+J19</f>
+        <v>2887392</v>
+      </c>
+      <c r="M19" s="41">
+        <f ca="1">L19/$L$22</f>
+        <v>0.15000057664716146</v>
+      </c>
+    </row>
+    <row r="20" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B20" s="34" t="s">
+        <v>76</v>
+      </c>
+      <c r="D20" s="12"/>
+      <c r="E20" s="1"/>
+      <c r="I20" s="6">
+        <v>3000000</v>
+      </c>
+      <c r="J20" s="22">
+        <f ca="1">IFERROR(ROUND(I20/$J$24,0),0)</f>
+        <v>721848</v>
+      </c>
+      <c r="L20" s="22">
+        <f ca="1">C20+E20+G20+J20</f>
+        <v>721848</v>
+      </c>
+      <c r="M20" s="41">
+        <f ca="1">L20/$L$22</f>
+        <v>3.7500144161790365E-2</v>
+      </c>
+    </row>
+    <row r="21" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B21" s="14"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="1"/>
+      <c r="I21" s="12"/>
+      <c r="J21" s="1"/>
+      <c r="L21" s="22"/>
+      <c r="M21" s="41"/>
+    </row>
+    <row r="22" spans="2:13" ht="13.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="44" t="s">
+        <v>68</v>
+      </c>
+      <c r="C22" s="47">
+        <f>C13</f>
+        <v>9675158</v>
+      </c>
+      <c r="D22" s="48">
+        <f>SUM(D15:D21)</f>
+        <v>9825000</v>
+      </c>
+      <c r="E22" s="47">
+        <f ca="1">SUM(E15:E21)</f>
+        <v>2836807</v>
+      </c>
+      <c r="F22" s="49"/>
+      <c r="G22" s="49">
+        <f ca="1">G13</f>
+        <v>1924921</v>
+      </c>
+      <c r="H22" s="49"/>
+      <c r="I22" s="48">
+        <f>SUM(I15:I21)</f>
+        <v>20000000</v>
+      </c>
+      <c r="J22" s="47">
+        <f ca="1">SUM(J15:J21)</f>
+        <v>4812320</v>
+      </c>
+      <c r="K22" s="49"/>
+      <c r="L22" s="47">
+        <f ca="1">C22+E22+G22+J22</f>
+        <v>19249206</v>
+      </c>
+      <c r="M22" s="50">
+        <f ca="1">SUM(M15:M20)+M13</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="2:13" ht="13.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="24" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B24" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="E24" s="52">
+        <f ca="1">IFERROR(ROUND($C$29/(C22+E22+G22),4),0)</f>
+        <v>3.4634</v>
+      </c>
+      <c r="J24" s="52">
+        <f ca="1">IFERROR(ROUND($C$30/(C22+E22+G22),4),0)</f>
+        <v>4.1559999999999997</v>
+      </c>
+    </row>
+    <row r="25" spans="2:13" ht="13.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B25" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="E25" s="51">
+        <f>C29</f>
+        <v>50000000</v>
+      </c>
+      <c r="J25" s="51">
+        <f>C30</f>
+        <v>60000000</v>
+      </c>
+    </row>
+    <row r="26" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B26" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="E26" s="51">
+        <f>C29</f>
+        <v>50000000</v>
+      </c>
+      <c r="J26" s="51">
+        <f>C30+C31</f>
+        <v>80000000</v>
+      </c>
+    </row>
+    <row r="28" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B28" s="23" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="29" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B29" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="C29" s="3">
+        <v>50000000</v>
+      </c>
+    </row>
+    <row r="30" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B30" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="C30" s="3">
+        <v>60000000</v>
+      </c>
+    </row>
+    <row r="31" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B31" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="C31" s="3">
+        <v>20000000</v>
+      </c>
+    </row>
+    <row r="32" spans="2:13" x14ac:dyDescent="0.2">
+      <c r="B32" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="C32" s="4">
+        <v>0.1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>